<commit_message>
Improve northern warming comparison pages
</commit_message>
<xml_diff>
--- a/data/tables/northern_warming/tables/northwest_territories_warming_tables.xlsx
+++ b/data/tables/northern_warming/tables/northwest_territories_warming_tables.xlsx
@@ -11,6 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Average comparison full" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faster areas report" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faster areas full" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annual reference series" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Year completeness" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -449,7 +451,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Compared with global surface</t>
+          <t>Compared with global average</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -476,11 +478,11 @@
         <v>2025</v>
       </c>
       <c r="C2" t="n">
-        <v>0.261551583002186</v>
+        <v>0.2638805455586553</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.8× faster</t>
+          <t>1.9× faster</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -507,7 +509,7 @@
         <v>2025</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3651406742105301</v>
+        <v>0.3672839573063428</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -538,7 +540,7 @@
         <v>2025</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4329685069595599</v>
+        <v>0.4360245424264593</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -569,7 +571,7 @@
         <v>2025</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4642583850483677</v>
+        <v>0.4680481211802833</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -600,7 +602,7 @@
         <v>2025</v>
       </c>
       <c r="C6" t="n">
-        <v>0.4748266349645389</v>
+        <v>0.4795372483656996</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -631,7 +633,7 @@
         <v>2025</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5361404204752027</v>
+        <v>0.5415477130413764</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -686,7 +688,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Compared with global surface</t>
+          <t>Compared with global average</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -706,7 +708,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Global surface rate (°C/decade)</t>
+          <t>Global average rate (°C/decade)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -733,11 +735,11 @@
         <v>2025</v>
       </c>
       <c r="C2" t="n">
-        <v>0.261551583002186</v>
+        <v>0.2638805455586553</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.8× faster</t>
+          <t>1.9× faster</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -762,10 +764,10 @@
         <v>0.2208353673690072</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2199353059175402</v>
+        <v>0.2193122683420462</v>
       </c>
       <c r="K2" t="n">
-        <v>0.2330057991078904</v>
+        <v>0.2323150399017823</v>
       </c>
     </row>
     <row r="3">
@@ -776,7 +778,7 @@
         <v>2025</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3651406742105301</v>
+        <v>0.3672839573063428</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -805,10 +807,10 @@
         <v>0.2570259324213248</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2803718469695279</v>
+        <v>0.2799826390854742</v>
       </c>
       <c r="K3" t="n">
-        <v>0.3078363719942164</v>
+        <v>0.3070893001596213</v>
       </c>
     </row>
     <row r="4">
@@ -819,7 +821,7 @@
         <v>2025</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4329685069595599</v>
+        <v>0.4360245424264593</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -848,10 +850,10 @@
         <v>0.2897269249773123</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3262311345338185</v>
+        <v>0.325175709998213</v>
       </c>
       <c r="K4" t="n">
-        <v>0.3630625906548526</v>
+        <v>0.361690648022655</v>
       </c>
     </row>
     <row r="5">
@@ -862,7 +864,7 @@
         <v>2025</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4642583850483677</v>
+        <v>0.4680481211802833</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -891,10 +893,10 @@
         <v>0.3280053462325782</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3773053526322572</v>
+        <v>0.375455574822453</v>
       </c>
       <c r="K5" t="n">
-        <v>0.4284884671324073</v>
+        <v>0.4264541436489675</v>
       </c>
     </row>
     <row r="6">
@@ -905,7 +907,7 @@
         <v>2025</v>
       </c>
       <c r="C6" t="n">
-        <v>0.4748266349645389</v>
+        <v>0.4795372483656996</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -934,10 +936,10 @@
         <v>0.3343533519136058</v>
       </c>
       <c r="J6" t="n">
-        <v>0.345252011259643</v>
+        <v>0.3429550470459525</v>
       </c>
       <c r="K6" t="n">
-        <v>0.4115433921836178</v>
+        <v>0.4090867065865657</v>
       </c>
     </row>
     <row r="7">
@@ -948,7 +950,7 @@
         <v>2025</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5361404204752027</v>
+        <v>0.5415477130413764</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -977,10 +979,10 @@
         <v>0.3762561489730054</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4264284414742858</v>
+        <v>0.4239276655602184</v>
       </c>
       <c r="K7" t="n">
-        <v>0.4972086611384779</v>
+        <v>0.4944605489941047</v>
       </c>
     </row>
   </sheetData>
@@ -1010,12 +1012,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Faster-warming Northwest Territories areas, 95th percentile (°C/decade)</t>
+          <t>Fastest-warming areas in Northwest Territories</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Compared with global surface</t>
+          <t>Compared with global average</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1042,11 +1044,11 @@
         <v>2025</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3621949347326592</v>
+        <v>0.3628835923183087</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.5× faster</t>
+          <t>2.6× faster</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1056,7 +1058,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.6× faster</t>
+          <t>1.7× faster</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1073,7 +1075,7 @@
         <v>2025</v>
       </c>
       <c r="C3" t="n">
-        <v>0.4866650513034746</v>
+        <v>0.4872202833980782</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1104,7 +1106,7 @@
         <v>2025</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5688555002008339</v>
+        <v>0.5695596495311227</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1118,7 +1120,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.7× faster</t>
+          <t>1.8× faster</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1135,7 +1137,7 @@
         <v>2025</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6775109886440015</v>
+        <v>0.6772588799520781</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1166,7 +1168,7 @@
         <v>2025</v>
       </c>
       <c r="C6" t="n">
-        <v>0.761379575585437</v>
+        <v>0.7608640450321417</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1197,7 +1199,7 @@
         <v>2025</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8026145733848598</v>
+        <v>0.8034535921860524</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1247,12 +1249,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Faster-warming Northwest Territories areas, 95th percentile (°C/decade)</t>
+          <t>Fastest-warming areas in Northwest Territories</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Compared with global surface</t>
+          <t>Compared with global average</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1272,7 +1274,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Global surface rate (°C/decade)</t>
+          <t>Global average rate (°C/decade)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -1304,11 +1306,11 @@
         <v>2025</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3621949347326592</v>
+        <v>0.3628835923183087</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.5× faster</t>
+          <t>2.6× faster</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1318,7 +1320,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1.6× faster</t>
+          <t>1.7× faster</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1333,10 +1335,10 @@
         <v>0.2208353673690072</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2199353059175402</v>
+        <v>0.2193122683420462</v>
       </c>
       <c r="K2" t="n">
-        <v>0.2330057991078904</v>
+        <v>0.2323150399017823</v>
       </c>
       <c r="L2" t="n">
         <v>95</v>
@@ -1350,7 +1352,7 @@
         <v>2025</v>
       </c>
       <c r="C3" t="n">
-        <v>0.4866650513034746</v>
+        <v>0.4872202833980782</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1379,10 +1381,10 @@
         <v>0.2570259324213248</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2803718469695279</v>
+        <v>0.2799826390854742</v>
       </c>
       <c r="K3" t="n">
-        <v>0.3078363719942164</v>
+        <v>0.3070893001596213</v>
       </c>
       <c r="L3" t="n">
         <v>95</v>
@@ -1396,7 +1398,7 @@
         <v>2025</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5688555002008339</v>
+        <v>0.5695596495311227</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1410,7 +1412,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1.7× faster</t>
+          <t>1.8× faster</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1425,10 +1427,10 @@
         <v>0.2897269249773123</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3262311345338185</v>
+        <v>0.325175709998213</v>
       </c>
       <c r="K4" t="n">
-        <v>0.3630625906548526</v>
+        <v>0.361690648022655</v>
       </c>
       <c r="L4" t="n">
         <v>95</v>
@@ -1442,7 +1444,7 @@
         <v>2025</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6775109886440015</v>
+        <v>0.6772588799520781</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1471,10 +1473,10 @@
         <v>0.3280053462325782</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3773053526322572</v>
+        <v>0.375455574822453</v>
       </c>
       <c r="K5" t="n">
-        <v>0.4284884671324073</v>
+        <v>0.4264541436489675</v>
       </c>
       <c r="L5" t="n">
         <v>95</v>
@@ -1488,7 +1490,7 @@
         <v>2025</v>
       </c>
       <c r="C6" t="n">
-        <v>0.761379575585437</v>
+        <v>0.7608640450321417</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1517,10 +1519,10 @@
         <v>0.3343533519136058</v>
       </c>
       <c r="J6" t="n">
-        <v>0.345252011259643</v>
+        <v>0.3429550470459525</v>
       </c>
       <c r="K6" t="n">
-        <v>0.4115433921836178</v>
+        <v>0.4090867065865657</v>
       </c>
       <c r="L6" t="n">
         <v>95</v>
@@ -1534,7 +1536,7 @@
         <v>2025</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8026145733848598</v>
+        <v>0.8034535921860524</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1563,13 +1565,4071 @@
         <v>0.3762561489730054</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4264284414742858</v>
+        <v>0.4239276655602184</v>
       </c>
       <c r="K7" t="n">
-        <v>0.4972086611384779</v>
+        <v>0.4944605489941047</v>
       </c>
       <c r="L7" t="n">
         <v>95</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J87"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Global average</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Global land</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Southern Canada</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Yukon</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Rest of Canada excluding Yukon</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Northwest Territories</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Rest of Canada excluding Northwest Territories</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Nunavut</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Rest of Canada excluding Nunavut</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1940</v>
+      </c>
+      <c r="B2" t="n">
+        <v>13.69043057564458</v>
+      </c>
+      <c r="C2" t="n">
+        <v>8.011690884027798</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-0.3326529592866357</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-5.617937105008365</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-3.885401586526421</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-6.908876100920765</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-3.532892436261493</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-12.55784696066569</v>
+      </c>
+      <c r="J2" t="n">
+        <v>-1.744598331434246</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1941</v>
+      </c>
+      <c r="B3" t="n">
+        <v>13.73878407089074</v>
+      </c>
+      <c r="C3" t="n">
+        <v>8.183946255132463</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-0.1905575050200881</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-6.286133709888288</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-4.494479020680481</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-8.966956180702176</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-3.928557815872991</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-14.48899569731733</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-2.01437020000819</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1942</v>
+      </c>
+      <c r="B4" t="n">
+        <v>13.64891403451929</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8.109579213069086</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.2103798882965486</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-5.796472485582477</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-4.143038916939163</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-8.037593972541995</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-3.655624349808861</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-13.39679293485185</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-1.846405098686195</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1943</v>
+      </c>
+      <c r="B5" t="n">
+        <v>13.65366753361602</v>
+      </c>
+      <c r="C5" t="n">
+        <v>8.185407421028536</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.3772654547579293</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-5.227543870698989</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-4.078150245255333</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-7.08713584774268</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-3.694181875549577</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-13.20100543538609</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-1.783638230317212</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1944</v>
+      </c>
+      <c r="B6" t="n">
+        <v>13.84095510596814</v>
+      </c>
+      <c r="C6" t="n">
+        <v>8.41790385075349</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.4350702945745796</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-4.769598075992053</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-3.496217839006618</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-6.981156860662179</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-3.048180051600821</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-13.00467846953944</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-1.109484892771609</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1945</v>
+      </c>
+      <c r="B7" t="n">
+        <v>13.7070656102983</v>
+      </c>
+      <c r="C7" t="n">
+        <v>8.106175190026693</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-1.153032981796486</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-6.511474889676211</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-4.923543510224274</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-8.894406776134446</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-4.420933353117992</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-13.64609227209801</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-2.760604450949283</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1946</v>
+      </c>
+      <c r="B8" t="n">
+        <v>13.7090479413186</v>
+      </c>
+      <c r="C8" t="n">
+        <v>8.185659112404654</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-0.79323259784954</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-6.641561732652055</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-4.707211166507914</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-8.834030756740571</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-4.201241010730469</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-13.75857962049764</v>
+      </c>
+      <c r="J8" t="n">
+        <v>-2.480837684128621</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1947</v>
+      </c>
+      <c r="B9" t="n">
+        <v>13.75378213968676</v>
+      </c>
+      <c r="C9" t="n">
+        <v>8.236751371071195</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-0.6510887934858871</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-5.85894497454583</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-4.231297916907389</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-8.578185174775891</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-3.674711721199686</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-12.14942528640606</v>
+      </c>
+      <c r="J9" t="n">
+        <v>-2.279592690282358</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1948</v>
+      </c>
+      <c r="B10" t="n">
+        <v>13.68855663720653</v>
+      </c>
+      <c r="C10" t="n">
+        <v>8.176407852228916</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-0.8170015965818799</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-8.517503339726757</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-4.859119693020497</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-9.227912324237128</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-4.416359465991782</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-14.13930426646359</v>
+      </c>
+      <c r="J10" t="n">
+        <v>-2.682290798808046</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1949</v>
+      </c>
+      <c r="B11" t="n">
+        <v>13.72586943551582</v>
+      </c>
+      <c r="C11" t="n">
+        <v>8.190172609171192</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-1.03165884283921</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-6.903343529436423</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-4.930610192284783</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-8.024864648902636</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-4.581361067301268</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-14.58957811559768</v>
+      </c>
+      <c r="J11" t="n">
+        <v>-2.549006523271947</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1950</v>
+      </c>
+      <c r="B12" t="n">
+        <v>13.61467633330517</v>
+      </c>
+      <c r="C12" t="n">
+        <v>7.935410504753428</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-2.177027189220774</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-7.097496400210535</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-5.878048782021178</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-9.176203231425831</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-5.454850403819987</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-14.8186183228077</v>
+      </c>
+      <c r="J12" t="n">
+        <v>-3.635260448448364</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1951</v>
+      </c>
+      <c r="B13" t="n">
+        <v>13.74845288205021</v>
+      </c>
+      <c r="C13" t="n">
+        <v>8.149450338215479</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-1.346006348084203</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-7.295192707852687</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-5.295195524197896</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-9.349389951281733</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-4.803878174977946</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-14.49733010151837</v>
+      </c>
+      <c r="J13" t="n">
+        <v>-3.033849692436357</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1952</v>
+      </c>
+      <c r="B14" t="n">
+        <v>13.72560247225752</v>
+      </c>
+      <c r="C14" t="n">
+        <v>8.035272161708857</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.1722462764292237</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-6.553438664965602</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-3.879035812337658</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-7.870174389355315</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-3.43604386269274</v>
+      </c>
+      <c r="I14" t="n">
+        <v>-13.42511429459409</v>
+      </c>
+      <c r="J14" t="n">
+        <v>-1.571051825635756</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1953</v>
+      </c>
+      <c r="B15" t="n">
+        <v>13.80752023492195</v>
+      </c>
+      <c r="C15" t="n">
+        <v>8.334412993306447</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.2347795141871966</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-6.255079734597619</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-3.869708282530267</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-7.553280229128206</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-3.456071812078446</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-13.7685882106397</v>
+      </c>
+      <c r="J15" t="n">
+        <v>-1.451922628900755</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>1954</v>
+      </c>
+      <c r="B16" t="n">
+        <v>13.61034425644664</v>
+      </c>
+      <c r="C16" t="n">
+        <v>8.049068671152671</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-0.6628160976511045</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-6.795196785597828</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-4.564602187788981</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-8.23027806313323</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-4.144718282002378</v>
+      </c>
+      <c r="I16" t="n">
+        <v>-13.87099732882011</v>
+      </c>
+      <c r="J16" t="n">
+        <v>-2.290771677365937</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>1955</v>
+      </c>
+      <c r="B17" t="n">
+        <v>13.59340965381186</v>
+      </c>
+      <c r="C17" t="n">
+        <v>8.14187734084639</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-0.6810330503840414</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-8.047355003780767</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-4.657766111225762</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-9.355172114498147</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-4.15033366451888</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-13.53557339231644</v>
+      </c>
+      <c r="J17" t="n">
+        <v>-2.568361705328901</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>1956</v>
+      </c>
+      <c r="B18" t="n">
+        <v>13.52870770667274</v>
+      </c>
+      <c r="C18" t="n">
+        <v>7.849739390896374</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-1.385824290000767</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-7.870562721848213</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-5.509610392364923</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-9.645141578602971</v>
+      </c>
+      <c r="H18" t="n">
+        <v>-5.026936952880121</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-15.1804325240264</v>
+      </c>
+      <c r="J18" t="n">
+        <v>-3.149456660520711</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1957</v>
+      </c>
+      <c r="B19" t="n">
+        <v>13.78207114754643</v>
+      </c>
+      <c r="C19" t="n">
+        <v>8.225985666889731</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-0.7677594865095184</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-5.320094771529793</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-4.797595285828823</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-8.713270203851653</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-4.241804387373753</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-14.32746827773397</v>
+      </c>
+      <c r="J19" t="n">
+        <v>-2.357869469433884</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1958</v>
+      </c>
+      <c r="B20" t="n">
+        <v>13.84805935178077</v>
+      </c>
+      <c r="C20" t="n">
+        <v>8.380354078559543</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-0.02886261013903971</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-5.722254964614196</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-4.094263713639845</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-8.187983783541076</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-3.575579984064392</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-13.61758910115648</v>
+      </c>
+      <c r="J20" t="n">
+        <v>-1.726076364405549</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>1959</v>
+      </c>
+      <c r="B21" t="n">
+        <v>13.81318674584848</v>
+      </c>
+      <c r="C21" t="n">
+        <v>8.323354789294006</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-0.9445410986697892</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-7.586690236102412</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-5.00794958857106</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-9.697564090494694</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-4.454924918763251</v>
+      </c>
+      <c r="I21" t="n">
+        <v>-14.14886113107107</v>
+      </c>
+      <c r="J21" t="n">
+        <v>-2.799051590708066</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1960</v>
+      </c>
+      <c r="B22" t="n">
+        <v>13.76304280509798</v>
+      </c>
+      <c r="C22" t="n">
+        <v>8.172513567636624</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-0.3097222048625001</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-6.486313811453701</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-4.249703459084006</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-8.731492039892313</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-3.70804760574311</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-13.15426176354247</v>
+      </c>
+      <c r="J22" t="n">
+        <v>-2.0805183838937</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>1961</v>
+      </c>
+      <c r="B23" t="n">
+        <v>13.84279138886267</v>
+      </c>
+      <c r="C23" t="n">
+        <v>8.376774708212775</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-0.2117103289607526</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-8.050267558927416</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-4.746332988461269</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-9.995964549646828</v>
+      </c>
+      <c r="H23" t="n">
+        <v>-4.151329075181938</v>
+      </c>
+      <c r="I23" t="n">
+        <v>-14.93704727757283</v>
+      </c>
+      <c r="J23" t="n">
+        <v>-2.310854815200494</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>1962</v>
+      </c>
+      <c r="B24" t="n">
+        <v>13.78246811576126</v>
+      </c>
+      <c r="C24" t="n">
+        <v>8.325135007353035</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-0.8072732988162884</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-6.309807030078508</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-4.679710182788313</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-8.388688518115421</v>
+      </c>
+      <c r="H24" t="n">
+        <v>-4.218718620943221</v>
+      </c>
+      <c r="I24" t="n">
+        <v>-13.87132436945424</v>
+      </c>
+      <c r="J24" t="n">
+        <v>-2.397725608407864</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>1963</v>
+      </c>
+      <c r="B25" t="n">
+        <v>13.81946226871661</v>
+      </c>
+      <c r="C25" t="n">
+        <v>8.415733425862536</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-0.5155131683942684</v>
+      </c>
+      <c r="E25" t="n">
+        <v>-6.319769381619277</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-4.445006083296494</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-8.265735457729138</v>
+      </c>
+      <c r="H25" t="n">
+        <v>-3.98140153207251</v>
+      </c>
+      <c r="I25" t="n">
+        <v>-13.73597125251535</v>
+      </c>
+      <c r="J25" t="n">
+        <v>-2.152699541616643</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>1964</v>
+      </c>
+      <c r="B26" t="n">
+        <v>13.60333128437458</v>
+      </c>
+      <c r="C26" t="n">
+        <v>8.023429813772184</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-1.007449437201353</v>
+      </c>
+      <c r="E26" t="n">
+        <v>-8.204611051430676</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-5.192391385550538</v>
+      </c>
+      <c r="G26" t="n">
+        <v>-9.399836836683603</v>
+      </c>
+      <c r="H26" t="n">
+        <v>-4.736512834051524</v>
+      </c>
+      <c r="I26" t="n">
+        <v>-14.99994505384998</v>
+      </c>
+      <c r="J26" t="n">
+        <v>-2.837903530597849</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>1965</v>
+      </c>
+      <c r="B27" t="n">
+        <v>13.67094742700516</v>
+      </c>
+      <c r="C27" t="n">
+        <v>8.152862461762012</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-1.50479333529286</v>
+      </c>
+      <c r="E27" t="n">
+        <v>-7.415011101538058</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-5.296552526748044</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-9.091918530067588</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-4.850796068149831</v>
+      </c>
+      <c r="I27" t="n">
+        <v>-14.19327197636829</v>
+      </c>
+      <c r="J27" t="n">
+        <v>-3.121937164753367</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>1966</v>
+      </c>
+      <c r="B28" t="n">
+        <v>13.74815768230339</v>
+      </c>
+      <c r="C28" t="n">
+        <v>8.224824069412861</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-0.8201873242751556</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-8.312786618422731</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-4.868836333641093</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-9.654508001188264</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-4.351331058946736</v>
+      </c>
+      <c r="I28" t="n">
+        <v>-13.90509586323679</v>
+      </c>
+      <c r="J28" t="n">
+        <v>-2.741752299259611</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>1967</v>
+      </c>
+      <c r="B29" t="n">
+        <v>13.7634132530287</v>
+      </c>
+      <c r="C29" t="n">
+        <v>8.262825607848763</v>
+      </c>
+      <c r="D29" t="n">
+        <v>-1.184187030358838</v>
+      </c>
+      <c r="E29" t="n">
+        <v>-6.619768368000371</v>
+      </c>
+      <c r="F29" t="n">
+        <v>-5.228688592537585</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-9.230870319958564</v>
+      </c>
+      <c r="H29" t="n">
+        <v>-4.710040525622419</v>
+      </c>
+      <c r="I29" t="n">
+        <v>-14.74759287591307</v>
+      </c>
+      <c r="J29" t="n">
+        <v>-2.846681490829472</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>1968</v>
+      </c>
+      <c r="B30" t="n">
+        <v>13.695035187117</v>
+      </c>
+      <c r="C30" t="n">
+        <v>8.123353720947794</v>
+      </c>
+      <c r="D30" t="n">
+        <v>-0.5450112004398701</v>
+      </c>
+      <c r="E30" t="n">
+        <v>-6.55185606762372</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-4.525625331876787</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-8.655449683936501</v>
+      </c>
+      <c r="H30" t="n">
+        <v>-4.024503890227293</v>
+      </c>
+      <c r="I30" t="n">
+        <v>-13.77358399004591</v>
+      </c>
+      <c r="J30" t="n">
+        <v>-2.254046743444812</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>1969</v>
+      </c>
+      <c r="B31" t="n">
+        <v>13.8312038334572</v>
+      </c>
+      <c r="C31" t="n">
+        <v>8.213444446430842</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-0.4802128268041829</v>
+      </c>
+      <c r="E31" t="n">
+        <v>-6.326723914046503</v>
+      </c>
+      <c r="F31" t="n">
+        <v>-4.19848938881894</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-7.952766473280248</v>
+      </c>
+      <c r="H31" t="n">
+        <v>-3.759444998477907</v>
+      </c>
+      <c r="I31" t="n">
+        <v>-12.90228422993901</v>
+      </c>
+      <c r="J31" t="n">
+        <v>-2.074550148657295</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>1970</v>
+      </c>
+      <c r="B32" t="n">
+        <v>13.80381375678246</v>
+      </c>
+      <c r="C32" t="n">
+        <v>8.344194338117621</v>
+      </c>
+      <c r="D32" t="n">
+        <v>-0.9403054837497881</v>
+      </c>
+      <c r="E32" t="n">
+        <v>-6.406578453318168</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-4.859589462438574</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-8.703259451977074</v>
+      </c>
+      <c r="H32" t="n">
+        <v>-4.373650873986201</v>
+      </c>
+      <c r="I32" t="n">
+        <v>-14.10565150147247</v>
+      </c>
+      <c r="J32" t="n">
+        <v>-2.558226850651214</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>1971</v>
+      </c>
+      <c r="B33" t="n">
+        <v>13.65070870843836</v>
+      </c>
+      <c r="C33" t="n">
+        <v>8.251643007445134</v>
+      </c>
+      <c r="D33" t="n">
+        <v>-0.6759595449608697</v>
+      </c>
+      <c r="E33" t="n">
+        <v>-7.889395314873724</v>
+      </c>
+      <c r="F33" t="n">
+        <v>-4.589319016973003</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-8.74218573224392</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-4.158206786858613</v>
+      </c>
+      <c r="I33" t="n">
+        <v>-13.62238711903773</v>
+      </c>
+      <c r="J33" t="n">
+        <v>-2.453973815720463</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>1972</v>
+      </c>
+      <c r="B34" t="n">
+        <v>13.78198341342426</v>
+      </c>
+      <c r="C34" t="n">
+        <v>8.150958367031723</v>
+      </c>
+      <c r="D34" t="n">
+        <v>-2.566915333819982</v>
+      </c>
+      <c r="E34" t="n">
+        <v>-8.216371980448374</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-6.694424007875527</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-10.2009017812902</v>
+      </c>
+      <c r="H34" t="n">
+        <v>-6.257497097568536</v>
+      </c>
+      <c r="I34" t="n">
+        <v>-16.77376245852604</v>
+      </c>
+      <c r="J34" t="n">
+        <v>-4.175267568233283</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>1973</v>
+      </c>
+      <c r="B35" t="n">
+        <v>13.88761343950328</v>
+      </c>
+      <c r="C35" t="n">
+        <v>8.589287371277686</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.07229780815960817</v>
+      </c>
+      <c r="E35" t="n">
+        <v>-7.164077820105703</v>
+      </c>
+      <c r="F35" t="n">
+        <v>-3.797038779345671</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-7.393774794022709</v>
+      </c>
+      <c r="H35" t="n">
+        <v>-3.453004498659019</v>
+      </c>
+      <c r="I35" t="n">
+        <v>-13.05033130537828</v>
+      </c>
+      <c r="J35" t="n">
+        <v>-1.608781894034158</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>1974</v>
+      </c>
+      <c r="B36" t="n">
+        <v>13.61420722376732</v>
+      </c>
+      <c r="C36" t="n">
+        <v>8.002236108952145</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-1.237721589227154</v>
+      </c>
+      <c r="E36" t="n">
+        <v>-7.385035148704995</v>
+      </c>
+      <c r="F36" t="n">
+        <v>-5.453215098958338</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-10.08534012918338</v>
+      </c>
+      <c r="H36" t="n">
+        <v>-4.871487747891503</v>
+      </c>
+      <c r="I36" t="n">
+        <v>-15.08346618762401</v>
+      </c>
+      <c r="J36" t="n">
+        <v>-3.076477942333314</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>1975</v>
+      </c>
+      <c r="B37" t="n">
+        <v>13.63716264439821</v>
+      </c>
+      <c r="C37" t="n">
+        <v>8.265033478330494</v>
+      </c>
+      <c r="D37" t="n">
+        <v>-0.7736300103879947</v>
+      </c>
+      <c r="E37" t="n">
+        <v>-7.433699756938429</v>
+      </c>
+      <c r="F37" t="n">
+        <v>-4.750551476218269</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-8.926373883549839</v>
+      </c>
+      <c r="H37" t="n">
+        <v>-4.280428712066823</v>
+      </c>
+      <c r="I37" t="n">
+        <v>-13.95844974599219</v>
+      </c>
+      <c r="J37" t="n">
+        <v>-2.530868263466143</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>1976</v>
+      </c>
+      <c r="B38" t="n">
+        <v>13.56440519112469</v>
+      </c>
+      <c r="C38" t="n">
+        <v>7.879184523090127</v>
+      </c>
+      <c r="D38" t="n">
+        <v>-0.7226998836723107</v>
+      </c>
+      <c r="E38" t="n">
+        <v>-5.448740521356766</v>
+      </c>
+      <c r="F38" t="n">
+        <v>-4.752860334055772</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-7.89629803792097</v>
+      </c>
+      <c r="H38" t="n">
+        <v>-4.322621099229462</v>
+      </c>
+      <c r="I38" t="n">
+        <v>-14.77158987386917</v>
+      </c>
+      <c r="J38" t="n">
+        <v>-2.197243296036563</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>1977</v>
+      </c>
+      <c r="B39" t="n">
+        <v>13.85508062118923</v>
+      </c>
+      <c r="C39" t="n">
+        <v>8.383890645727373</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.2033718656115622</v>
+      </c>
+      <c r="E39" t="n">
+        <v>-5.459178507232486</v>
+      </c>
+      <c r="F39" t="n">
+        <v>-3.737819564509649</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-7.836428418057293</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-3.223788412813117</v>
+      </c>
+      <c r="I39" t="n">
+        <v>-12.88807064771115</v>
+      </c>
+      <c r="J39" t="n">
+        <v>-1.472333046990349</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>1978</v>
+      </c>
+      <c r="B40" t="n">
+        <v>13.79599116635706</v>
+      </c>
+      <c r="C40" t="n">
+        <v>8.247198056775574</v>
+      </c>
+      <c r="D40" t="n">
+        <v>-1.246338815524421</v>
+      </c>
+      <c r="E40" t="n">
+        <v>-5.157578075678276</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-5.310940744995991</v>
+      </c>
+      <c r="G40" t="n">
+        <v>-8.630330069186606</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-4.805400873592075</v>
+      </c>
+      <c r="I40" t="n">
+        <v>-15.3210977881994</v>
+      </c>
+      <c r="J40" t="n">
+        <v>-2.703897031159098</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>1979</v>
+      </c>
+      <c r="B41" t="n">
+        <v>13.95342295070824</v>
+      </c>
+      <c r="C41" t="n">
+        <v>8.401263366793479</v>
+      </c>
+      <c r="D41" t="n">
+        <v>-0.6732554052500564</v>
+      </c>
+      <c r="E41" t="n">
+        <v>-5.916064434805404</v>
+      </c>
+      <c r="F41" t="n">
+        <v>-4.803256122599149</v>
+      </c>
+      <c r="G41" t="n">
+        <v>-8.59021401163991</v>
+      </c>
+      <c r="H41" t="n">
+        <v>-4.300766319884153</v>
+      </c>
+      <c r="I41" t="n">
+        <v>-14.71281395174872</v>
+      </c>
+      <c r="J41" t="n">
+        <v>-2.302305555678712</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>1980</v>
+      </c>
+      <c r="B42" t="n">
+        <v>14.07790809274332</v>
+      </c>
+      <c r="C42" t="n">
+        <v>8.697190817270185</v>
+      </c>
+      <c r="D42" t="n">
+        <v>-0.4842241006869986</v>
+      </c>
+      <c r="E42" t="n">
+        <v>-6.056531908652018</v>
+      </c>
+      <c r="F42" t="n">
+        <v>-4.273756228687438</v>
+      </c>
+      <c r="G42" t="n">
+        <v>-7.986332133815951</v>
+      </c>
+      <c r="H42" t="n">
+        <v>-3.821030671573644</v>
+      </c>
+      <c r="I42" t="n">
+        <v>-13.2161475988962</v>
+      </c>
+      <c r="J42" t="n">
+        <v>-2.066083485373929</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>1981</v>
+      </c>
+      <c r="B43" t="n">
+        <v>14.11629583112865</v>
+      </c>
+      <c r="C43" t="n">
+        <v>8.888912599967027</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1.210247003543447</v>
+      </c>
+      <c r="E43" t="n">
+        <v>-4.130133946012435</v>
+      </c>
+      <c r="F43" t="n">
+        <v>-2.617985192813364</v>
+      </c>
+      <c r="G43" t="n">
+        <v>-5.984899709925047</v>
+      </c>
+      <c r="H43" t="n">
+        <v>-2.201376722002047</v>
+      </c>
+      <c r="I43" t="n">
+        <v>-11.89403757009172</v>
+      </c>
+      <c r="J43" t="n">
+        <v>-0.3066398940159317</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>1982</v>
+      </c>
+      <c r="B44" t="n">
+        <v>13.91712094370134</v>
+      </c>
+      <c r="C44" t="n">
+        <v>8.362596808060404</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-1.50289562012097</v>
+      </c>
+      <c r="E44" t="n">
+        <v>-7.654977450363557</v>
+      </c>
+      <c r="F44" t="n">
+        <v>-5.602223050645479</v>
+      </c>
+      <c r="G44" t="n">
+        <v>-10.06833964384435</v>
+      </c>
+      <c r="H44" t="n">
+        <v>-5.052310096162012</v>
+      </c>
+      <c r="I44" t="n">
+        <v>-14.99133009466598</v>
+      </c>
+      <c r="J44" t="n">
+        <v>-3.295696049660447</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>1983</v>
+      </c>
+      <c r="B45" t="n">
+        <v>14.11096790609288</v>
+      </c>
+      <c r="C45" t="n">
+        <v>8.738856444670766</v>
+      </c>
+      <c r="D45" t="n">
+        <v>-0.1845328916807096</v>
+      </c>
+      <c r="E45" t="n">
+        <v>-6.757452491608546</v>
+      </c>
+      <c r="F45" t="n">
+        <v>-4.482758068728223</v>
+      </c>
+      <c r="G45" t="n">
+        <v>-8.802426379293122</v>
+      </c>
+      <c r="H45" t="n">
+        <v>-3.967557190559396</v>
+      </c>
+      <c r="I45" t="n">
+        <v>-14.55684961560684</v>
+      </c>
+      <c r="J45" t="n">
+        <v>-2.012517882080567</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>1984</v>
+      </c>
+      <c r="B46" t="n">
+        <v>13.89532993274377</v>
+      </c>
+      <c r="C46" t="n">
+        <v>8.375720439317485</v>
+      </c>
+      <c r="D46" t="n">
+        <v>-0.2221425623810813</v>
+      </c>
+      <c r="E46" t="n">
+        <v>-6.015247963515188</v>
+      </c>
+      <c r="F46" t="n">
+        <v>-4.403384352627792</v>
+      </c>
+      <c r="G46" t="n">
+        <v>-8.540981602256235</v>
+      </c>
+      <c r="H46" t="n">
+        <v>-3.877205059573332</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-14.24404548417876</v>
+      </c>
+      <c r="J46" t="n">
+        <v>-1.95183841246688</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>1985</v>
+      </c>
+      <c r="B47" t="n">
+        <v>13.85986580938163</v>
+      </c>
+      <c r="C47" t="n">
+        <v>8.326186326237247</v>
+      </c>
+      <c r="D47" t="n">
+        <v>-0.8474040933769079</v>
+      </c>
+      <c r="E47" t="n">
+        <v>-5.861797331966567</v>
+      </c>
+      <c r="F47" t="n">
+        <v>-4.664059148174506</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-8.827284654854617</v>
+      </c>
+      <c r="H47" t="n">
+        <v>-4.110164158481973</v>
+      </c>
+      <c r="I47" t="n">
+        <v>-13.4025274770132</v>
+      </c>
+      <c r="J47" t="n">
+        <v>-2.472338915484085</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>1986</v>
+      </c>
+      <c r="B48" t="n">
+        <v>13.94697218635512</v>
+      </c>
+      <c r="C48" t="n">
+        <v>8.529983752026428</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-0.2514886508334715</v>
+      </c>
+      <c r="E48" t="n">
+        <v>-5.69263600100947</v>
+      </c>
+      <c r="F48" t="n">
+        <v>-4.684359021864764</v>
+      </c>
+      <c r="G48" t="n">
+        <v>-8.794076331318589</v>
+      </c>
+      <c r="H48" t="n">
+        <v>-4.127545313578775</v>
+      </c>
+      <c r="I48" t="n">
+        <v>-15.29216501186155</v>
+      </c>
+      <c r="J48" t="n">
+        <v>-1.995628863028345</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>1987</v>
+      </c>
+      <c r="B49" t="n">
+        <v>14.10282603145438</v>
+      </c>
+      <c r="C49" t="n">
+        <v>8.700475228206267</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1.34994300806786</v>
+      </c>
+      <c r="E49" t="n">
+        <v>-4.491478774437899</v>
+      </c>
+      <c r="F49" t="n">
+        <v>-3.126966091026226</v>
+      </c>
+      <c r="G49" t="n">
+        <v>-6.961809337551475</v>
+      </c>
+      <c r="H49" t="n">
+        <v>-2.631825672877163</v>
+      </c>
+      <c r="I49" t="n">
+        <v>-14.03961293348477</v>
+      </c>
+      <c r="J49" t="n">
+        <v>-0.3816435049083745</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>1988</v>
+      </c>
+      <c r="B50" t="n">
+        <v>14.13113825237433</v>
+      </c>
+      <c r="C50" t="n">
+        <v>8.907656175206741</v>
+      </c>
+      <c r="D50" t="n">
+        <v>-0.04835242697436799</v>
+      </c>
+      <c r="E50" t="n">
+        <v>-5.244413317114624</v>
+      </c>
+      <c r="F50" t="n">
+        <v>-4.012353079588922</v>
+      </c>
+      <c r="G50" t="n">
+        <v>-8.013232700734022</v>
+      </c>
+      <c r="H50" t="n">
+        <v>-3.484729885767596</v>
+      </c>
+      <c r="I50" t="n">
+        <v>-13.2922904800227</v>
+      </c>
+      <c r="J50" t="n">
+        <v>-1.682305107613606</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>1989</v>
+      </c>
+      <c r="B51" t="n">
+        <v>14.01638740546175</v>
+      </c>
+      <c r="C51" t="n">
+        <v>8.65657060190965</v>
+      </c>
+      <c r="D51" t="n">
+        <v>-0.9264306289894491</v>
+      </c>
+      <c r="E51" t="n">
+        <v>-5.203918069113596</v>
+      </c>
+      <c r="F51" t="n">
+        <v>-4.879616074402695</v>
+      </c>
+      <c r="G51" t="n">
+        <v>-8.225819497252258</v>
+      </c>
+      <c r="H51" t="n">
+        <v>-4.397608731272713</v>
+      </c>
+      <c r="I51" t="n">
+        <v>-14.54095399012429</v>
+      </c>
+      <c r="J51" t="n">
+        <v>-2.393257651929361</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>1990</v>
+      </c>
+      <c r="B52" t="n">
+        <v>14.24924986771015</v>
+      </c>
+      <c r="C52" t="n">
+        <v>8.974928186866773</v>
+      </c>
+      <c r="D52" t="n">
+        <v>-0.4754288929981274</v>
+      </c>
+      <c r="E52" t="n">
+        <v>-6.553305380178102</v>
+      </c>
+      <c r="F52" t="n">
+        <v>-4.824522049730618</v>
+      </c>
+      <c r="G52" t="n">
+        <v>-9.359064263114416</v>
+      </c>
+      <c r="H52" t="n">
+        <v>-4.245688235273335</v>
+      </c>
+      <c r="I52" t="n">
+        <v>-14.91438042316036</v>
+      </c>
+      <c r="J52" t="n">
+        <v>-2.315702828576911</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>1991</v>
+      </c>
+      <c r="B53" t="n">
+        <v>14.19236932713923</v>
+      </c>
+      <c r="C53" t="n">
+        <v>8.885097619611615</v>
+      </c>
+      <c r="D53" t="n">
+        <v>-0.0390618734019884</v>
+      </c>
+      <c r="E53" t="n">
+        <v>-5.3504422008765</v>
+      </c>
+      <c r="F53" t="n">
+        <v>-4.233234824218369</v>
+      </c>
+      <c r="G53" t="n">
+        <v>-8.500903506604265</v>
+      </c>
+      <c r="H53" t="n">
+        <v>-3.659067639785291</v>
+      </c>
+      <c r="I53" t="n">
+        <v>-14.03023678885707</v>
+      </c>
+      <c r="J53" t="n">
+        <v>-1.761767258765595</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>1992</v>
+      </c>
+      <c r="B54" t="n">
+        <v>13.95644895242778</v>
+      </c>
+      <c r="C54" t="n">
+        <v>8.470906583813663</v>
+      </c>
+      <c r="D54" t="n">
+        <v>-0.7546456587878561</v>
+      </c>
+      <c r="E54" t="n">
+        <v>-6.227099253412269</v>
+      </c>
+      <c r="F54" t="n">
+        <v>-4.844376250713757</v>
+      </c>
+      <c r="G54" t="n">
+        <v>-8.456318496632909</v>
+      </c>
+      <c r="H54" t="n">
+        <v>-4.383639686250285</v>
+      </c>
+      <c r="I54" t="n">
+        <v>-14.74455334233691</v>
+      </c>
+      <c r="J54" t="n">
+        <v>-2.362911608346532</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>1993</v>
+      </c>
+      <c r="B55" t="n">
+        <v>14.00688804708349</v>
+      </c>
+      <c r="C55" t="n">
+        <v>8.583487742832272</v>
+      </c>
+      <c r="D55" t="n">
+        <v>-0.4712216502193975</v>
+      </c>
+      <c r="E55" t="n">
+        <v>-4.010651929550618</v>
+      </c>
+      <c r="F55" t="n">
+        <v>-4.326304652582732</v>
+      </c>
+      <c r="G55" t="n">
+        <v>-7.015433514457242</v>
+      </c>
+      <c r="H55" t="n">
+        <v>-3.905715106819484</v>
+      </c>
+      <c r="I55" t="n">
+        <v>-14.11055424663235</v>
+      </c>
+      <c r="J55" t="n">
+        <v>-1.767624896524005</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>1994</v>
+      </c>
+      <c r="B56" t="n">
+        <v>14.04477926471139</v>
+      </c>
+      <c r="C56" t="n">
+        <v>8.755904775315386</v>
+      </c>
+      <c r="D56" t="n">
+        <v>-0.3150391664258419</v>
+      </c>
+      <c r="E56" t="n">
+        <v>-5.853600262471464</v>
+      </c>
+      <c r="F56" t="n">
+        <v>-4.123895693666395</v>
+      </c>
+      <c r="G56" t="n">
+        <v>-7.790098290571839</v>
+      </c>
+      <c r="H56" t="n">
+        <v>-3.675048815721987</v>
+      </c>
+      <c r="I56" t="n">
+        <v>-13.15314706412913</v>
+      </c>
+      <c r="J56" t="n">
+        <v>-1.890332443824283</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>1995</v>
+      </c>
+      <c r="B57" t="n">
+        <v>14.21911714260189</v>
+      </c>
+      <c r="C57" t="n">
+        <v>9.044514844715234</v>
+      </c>
+      <c r="D57" t="n">
+        <v>-0.2922674313945443</v>
+      </c>
+      <c r="E57" t="n">
+        <v>-5.278128322783035</v>
+      </c>
+      <c r="F57" t="n">
+        <v>-4.090187650314967</v>
+      </c>
+      <c r="G57" t="n">
+        <v>-7.730111716069859</v>
+      </c>
+      <c r="H57" t="n">
+        <v>-3.61403177975163</v>
+      </c>
+      <c r="I57" t="n">
+        <v>-13.10346527522928</v>
+      </c>
+      <c r="J57" t="n">
+        <v>-1.826543153753556</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>1996</v>
+      </c>
+      <c r="B58" t="n">
+        <v>14.08627927036392</v>
+      </c>
+      <c r="C58" t="n">
+        <v>8.692077179223393</v>
+      </c>
+      <c r="D58" t="n">
+        <v>-1.150548652493746</v>
+      </c>
+      <c r="E58" t="n">
+        <v>-7.67122726964273</v>
+      </c>
+      <c r="F58" t="n">
+        <v>-4.709340662128489</v>
+      </c>
+      <c r="G58" t="n">
+        <v>-8.573147739239548</v>
+      </c>
+      <c r="H58" t="n">
+        <v>-4.301979875939637</v>
+      </c>
+      <c r="I58" t="n">
+        <v>-12.86887630426572</v>
+      </c>
+      <c r="J58" t="n">
+        <v>-2.779287469684493</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>1997</v>
+      </c>
+      <c r="B59" t="n">
+        <v>14.21396009353637</v>
+      </c>
+      <c r="C59" t="n">
+        <v>8.833450567413729</v>
+      </c>
+      <c r="D59" t="n">
+        <v>-0.1847919496307432</v>
+      </c>
+      <c r="E59" t="n">
+        <v>-5.249456418884191</v>
+      </c>
+      <c r="F59" t="n">
+        <v>-4.077158609776562</v>
+      </c>
+      <c r="G59" t="n">
+        <v>-7.650812525153863</v>
+      </c>
+      <c r="H59" t="n">
+        <v>-3.610017002875422</v>
+      </c>
+      <c r="I59" t="n">
+        <v>-13.41363420828337</v>
+      </c>
+      <c r="J59" t="n">
+        <v>-1.728665063943308</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>1998</v>
+      </c>
+      <c r="B60" t="n">
+        <v>14.40097630563749</v>
+      </c>
+      <c r="C60" t="n">
+        <v>9.205549128702256</v>
+      </c>
+      <c r="D60" t="n">
+        <v>1.378348984312762</v>
+      </c>
+      <c r="E60" t="n">
+        <v>-4.963988220849564</v>
+      </c>
+      <c r="F60" t="n">
+        <v>-2.382009397938853</v>
+      </c>
+      <c r="G60" t="n">
+        <v>-5.51232772447942</v>
+      </c>
+      <c r="H60" t="n">
+        <v>-2.062496409186688</v>
+      </c>
+      <c r="I60" t="n">
+        <v>-11.60536321855317</v>
+      </c>
+      <c r="J60" t="n">
+        <v>-0.1519245130797496</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>1999</v>
+      </c>
+      <c r="B61" t="n">
+        <v>14.13149572585292</v>
+      </c>
+      <c r="C61" t="n">
+        <v>8.950350886701687</v>
+      </c>
+      <c r="D61" t="n">
+        <v>1.195861211541586</v>
+      </c>
+      <c r="E61" t="n">
+        <v>-6.078518802929861</v>
+      </c>
+      <c r="F61" t="n">
+        <v>-3.057836682167562</v>
+      </c>
+      <c r="G61" t="n">
+        <v>-7.242872003815041</v>
+      </c>
+      <c r="H61" t="n">
+        <v>-2.605799458681255</v>
+      </c>
+      <c r="I61" t="n">
+        <v>-13.08435337743479</v>
+      </c>
+      <c r="J61" t="n">
+        <v>-0.6470686790417941</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B62" t="n">
+        <v>14.12251664054831</v>
+      </c>
+      <c r="C62" t="n">
+        <v>8.808146153756283</v>
+      </c>
+      <c r="D62" t="n">
+        <v>-0.08135084802839247</v>
+      </c>
+      <c r="E62" t="n">
+        <v>-5.764723011427694</v>
+      </c>
+      <c r="F62" t="n">
+        <v>-3.979169120188657</v>
+      </c>
+      <c r="G62" t="n">
+        <v>-7.903023388382359</v>
+      </c>
+      <c r="H62" t="n">
+        <v>-3.494989177829085</v>
+      </c>
+      <c r="I62" t="n">
+        <v>-13.1106314729609</v>
+      </c>
+      <c r="J62" t="n">
+        <v>-1.722613273256315</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>2001</v>
+      </c>
+      <c r="B63" t="n">
+        <v>14.28915395293253</v>
+      </c>
+      <c r="C63" t="n">
+        <v>9.08596114694458</v>
+      </c>
+      <c r="D63" t="n">
+        <v>1.239415280566746</v>
+      </c>
+      <c r="E63" t="n">
+        <v>-5.201640071572075</v>
+      </c>
+      <c r="F63" t="n">
+        <v>-2.851171776216514</v>
+      </c>
+      <c r="G63" t="n">
+        <v>-6.888617540447905</v>
+      </c>
+      <c r="H63" t="n">
+        <v>-2.382570759070742</v>
+      </c>
+      <c r="I63" t="n">
+        <v>-12.4850724049836</v>
+      </c>
+      <c r="J63" t="n">
+        <v>-0.4999358090368883</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B64" t="n">
+        <v>14.38501333826196</v>
+      </c>
+      <c r="C64" t="n">
+        <v>9.267174959257533</v>
+      </c>
+      <c r="D64" t="n">
+        <v>-0.4576761390656653</v>
+      </c>
+      <c r="E64" t="n">
+        <v>-4.899224620218813</v>
+      </c>
+      <c r="F64" t="n">
+        <v>-4.211660223251681</v>
+      </c>
+      <c r="G64" t="n">
+        <v>-7.765797228964522</v>
+      </c>
+      <c r="H64" t="n">
+        <v>-3.719486550707018</v>
+      </c>
+      <c r="I64" t="n">
+        <v>-13.14826363439404</v>
+      </c>
+      <c r="J64" t="n">
+        <v>-1.936299215982701</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B65" t="n">
+        <v>14.3728158769447</v>
+      </c>
+      <c r="C65" t="n">
+        <v>9.216521340150363</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0.2273824884112743</v>
+      </c>
+      <c r="E65" t="n">
+        <v>-5.365397634765561</v>
+      </c>
+      <c r="F65" t="n">
+        <v>-3.560009767853565</v>
+      </c>
+      <c r="G65" t="n">
+        <v>-7.413232736306578</v>
+      </c>
+      <c r="H65" t="n">
+        <v>-3.087542464299833</v>
+      </c>
+      <c r="I65" t="n">
+        <v>-12.40716806371866</v>
+      </c>
+      <c r="J65" t="n">
+        <v>-1.378475863532569</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B66" t="n">
+        <v>14.30470323905453</v>
+      </c>
+      <c r="C66" t="n">
+        <v>9.026763455166556</v>
+      </c>
+      <c r="D66" t="n">
+        <v>-0.2966044438257777</v>
+      </c>
+      <c r="E66" t="n">
+        <v>-5.059236869780879</v>
+      </c>
+      <c r="F66" t="n">
+        <v>-4.771775779887533</v>
+      </c>
+      <c r="G66" t="n">
+        <v>-9.653864092866389</v>
+      </c>
+      <c r="H66" t="n">
+        <v>-4.057822174643942</v>
+      </c>
+      <c r="I66" t="n">
+        <v>-15.01761040061694</v>
+      </c>
+      <c r="J66" t="n">
+        <v>-2.131429427314042</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B67" t="n">
+        <v>14.47313817288972</v>
+      </c>
+      <c r="C67" t="n">
+        <v>9.43795712433538</v>
+      </c>
+      <c r="D67" t="n">
+        <v>1.030610573884831</v>
+      </c>
+      <c r="E67" t="n">
+        <v>-4.117509268712699</v>
+      </c>
+      <c r="F67" t="n">
+        <v>-3.079529853178447</v>
+      </c>
+      <c r="G67" t="n">
+        <v>-7.013894584447487</v>
+      </c>
+      <c r="H67" t="n">
+        <v>-2.550667801131761</v>
+      </c>
+      <c r="I67" t="n">
+        <v>-12.83679973094247</v>
+      </c>
+      <c r="J67" t="n">
+        <v>-0.6133664159803324</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B68" t="n">
+        <v>14.42411520384602</v>
+      </c>
+      <c r="C68" t="n">
+        <v>9.286630563005993</v>
+      </c>
+      <c r="D68" t="n">
+        <v>1.699621116550594</v>
+      </c>
+      <c r="E68" t="n">
+        <v>-5.514722970432989</v>
+      </c>
+      <c r="F68" t="n">
+        <v>-2.063199653948536</v>
+      </c>
+      <c r="G68" t="n">
+        <v>-5.740086156500277</v>
+      </c>
+      <c r="H68" t="n">
+        <v>-1.712043914047551</v>
+      </c>
+      <c r="I68" t="n">
+        <v>-10.94857351715988</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0.02425535467549584</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B69" t="n">
+        <v>14.41695814330639</v>
+      </c>
+      <c r="C69" t="n">
+        <v>9.472656279833451</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0.1891081808003666</v>
+      </c>
+      <c r="E69" t="n">
+        <v>-5.564293892679712</v>
+      </c>
+      <c r="F69" t="n">
+        <v>-3.82057220140158</v>
+      </c>
+      <c r="G69" t="n">
+        <v>-7.856413324650366</v>
+      </c>
+      <c r="H69" t="n">
+        <v>-3.317222848348476</v>
+      </c>
+      <c r="I69" t="n">
+        <v>-13.21448842504531</v>
+      </c>
+      <c r="J69" t="n">
+        <v>-1.493274182421768</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B70" t="n">
+        <v>14.28106556295393</v>
+      </c>
+      <c r="C70" t="n">
+        <v>9.143188597309269</v>
+      </c>
+      <c r="D70" t="n">
+        <v>-0.0898154995451273</v>
+      </c>
+      <c r="E70" t="n">
+        <v>-6.195238322078254</v>
+      </c>
+      <c r="F70" t="n">
+        <v>-4.050860869990824</v>
+      </c>
+      <c r="G70" t="n">
+        <v>-8.146615163248875</v>
+      </c>
+      <c r="H70" t="n">
+        <v>-3.561650503188024</v>
+      </c>
+      <c r="I70" t="n">
+        <v>-13.26205472399178</v>
+      </c>
+      <c r="J70" t="n">
+        <v>-1.796285647198106</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B71" t="n">
+        <v>14.41565621438641</v>
+      </c>
+      <c r="C71" t="n">
+        <v>9.256013601363724</v>
+      </c>
+      <c r="D71" t="n">
+        <v>-0.1047786439621025</v>
+      </c>
+      <c r="E71" t="n">
+        <v>-5.494888549191698</v>
+      </c>
+      <c r="F71" t="n">
+        <v>-3.871907817165033</v>
+      </c>
+      <c r="G71" t="n">
+        <v>-7.886999535608228</v>
+      </c>
+      <c r="H71" t="n">
+        <v>-3.36470068923002</v>
+      </c>
+      <c r="I71" t="n">
+        <v>-12.55644150876029</v>
+      </c>
+      <c r="J71" t="n">
+        <v>-1.721046848658403</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B72" t="n">
+        <v>14.51001282645987</v>
+      </c>
+      <c r="C72" t="n">
+        <v>9.468710411827946</v>
+      </c>
+      <c r="D72" t="n">
+        <v>2.038150291331934</v>
+      </c>
+      <c r="E72" t="n">
+        <v>-4.090300184796294</v>
+      </c>
+      <c r="F72" t="n">
+        <v>-1.541424429811114</v>
+      </c>
+      <c r="G72" t="n">
+        <v>-5.43879264590465</v>
+      </c>
+      <c r="H72" t="n">
+        <v>-1.105225184576916</v>
+      </c>
+      <c r="I72" t="n">
+        <v>-9.741662421776015</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0.4252818807988339</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B73" t="n">
+        <v>14.37030848032745</v>
+      </c>
+      <c r="C73" t="n">
+        <v>9.249171651857194</v>
+      </c>
+      <c r="D73" t="n">
+        <v>0.6242405824896694</v>
+      </c>
+      <c r="E73" t="n">
+        <v>-5.327474503639237</v>
+      </c>
+      <c r="F73" t="n">
+        <v>-3.244282938938259</v>
+      </c>
+      <c r="G73" t="n">
+        <v>-6.965426230656147</v>
+      </c>
+      <c r="H73" t="n">
+        <v>-2.807599084340745</v>
+      </c>
+      <c r="I73" t="n">
+        <v>-12.41655465834434</v>
+      </c>
+      <c r="J73" t="n">
+        <v>-0.9959414942240626</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B74" t="n">
+        <v>14.41598237324642</v>
+      </c>
+      <c r="C74" t="n">
+        <v>9.248810252234385</v>
+      </c>
+      <c r="D74" t="n">
+        <v>1.142947544559073</v>
+      </c>
+      <c r="E74" t="n">
+        <v>-6.022226870150861</v>
+      </c>
+      <c r="F74" t="n">
+        <v>-2.812726300311612</v>
+      </c>
+      <c r="G74" t="n">
+        <v>-6.671174893090277</v>
+      </c>
+      <c r="H74" t="n">
+        <v>-2.420446153419417</v>
+      </c>
+      <c r="I74" t="n">
+        <v>-12.15784657089829</v>
+      </c>
+      <c r="J74" t="n">
+        <v>-0.5906901827561727</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B75" t="n">
+        <v>14.44748933354398</v>
+      </c>
+      <c r="C75" t="n">
+        <v>9.387085708574924</v>
+      </c>
+      <c r="D75" t="n">
+        <v>0.0987622897893656</v>
+      </c>
+      <c r="E75" t="n">
+        <v>-4.899677222676853</v>
+      </c>
+      <c r="F75" t="n">
+        <v>-3.895311445035302</v>
+      </c>
+      <c r="G75" t="n">
+        <v>-7.698161598489341</v>
+      </c>
+      <c r="H75" t="n">
+        <v>-3.384190195936065</v>
+      </c>
+      <c r="I75" t="n">
+        <v>-13.38994054893918</v>
+      </c>
+      <c r="J75" t="n">
+        <v>-1.49517237798377</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B76" t="n">
+        <v>14.48824158723409</v>
+      </c>
+      <c r="C76" t="n">
+        <v>9.340143525392069</v>
+      </c>
+      <c r="D76" t="n">
+        <v>-0.2222100116732272</v>
+      </c>
+      <c r="E76" t="n">
+        <v>-4.237788479326875</v>
+      </c>
+      <c r="F76" t="n">
+        <v>-4.021197824159203</v>
+      </c>
+      <c r="G76" t="n">
+        <v>-7.45853199248258</v>
+      </c>
+      <c r="H76" t="n">
+        <v>-3.519342905478848</v>
+      </c>
+      <c r="I76" t="n">
+        <v>-13.16564919177821</v>
+      </c>
+      <c r="J76" t="n">
+        <v>-1.662152290440547</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B77" t="n">
+        <v>14.63674357729909</v>
+      </c>
+      <c r="C77" t="n">
+        <v>9.626736475286478</v>
+      </c>
+      <c r="D77" t="n">
+        <v>0.6916255165401095</v>
+      </c>
+      <c r="E77" t="n">
+        <v>-3.72487251386513</v>
+      </c>
+      <c r="F77" t="n">
+        <v>-3.418233868045584</v>
+      </c>
+      <c r="G77" t="n">
+        <v>-6.548304003739807</v>
+      </c>
+      <c r="H77" t="n">
+        <v>-2.967549014339067</v>
+      </c>
+      <c r="I77" t="n">
+        <v>-13.68280954302871</v>
+      </c>
+      <c r="J77" t="n">
+        <v>-0.7742362814161639</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B78" t="n">
+        <v>14.81423450213943</v>
+      </c>
+      <c r="C78" t="n">
+        <v>9.834334388164306</v>
+      </c>
+      <c r="D78" t="n">
+        <v>1.122079311476868</v>
+      </c>
+      <c r="E78" t="n">
+        <v>-3.18455830513801</v>
+      </c>
+      <c r="F78" t="n">
+        <v>-2.623297860097525</v>
+      </c>
+      <c r="G78" t="n">
+        <v>-5.939480078660049</v>
+      </c>
+      <c r="H78" t="n">
+        <v>-2.159447099908718</v>
+      </c>
+      <c r="I78" t="n">
+        <v>-11.68460046565566</v>
+      </c>
+      <c r="J78" t="n">
+        <v>-0.3076016449517641</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B79" t="n">
+        <v>14.72358098865754</v>
+      </c>
+      <c r="C79" t="n">
+        <v>9.695913720390354</v>
+      </c>
+      <c r="D79" t="n">
+        <v>0.6232090945763307</v>
+      </c>
+      <c r="E79" t="n">
+        <v>-4.348986911428898</v>
+      </c>
+      <c r="F79" t="n">
+        <v>-3.117740213638776</v>
+      </c>
+      <c r="G79" t="n">
+        <v>-6.116972608178957</v>
+      </c>
+      <c r="H79" t="n">
+        <v>-2.739951374913145</v>
+      </c>
+      <c r="I79" t="n">
+        <v>-12.36609826894861</v>
+      </c>
+      <c r="J79" t="n">
+        <v>-0.795834800613619</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B80" t="n">
+        <v>14.64448905881926</v>
+      </c>
+      <c r="C80" t="n">
+        <v>9.552322644933925</v>
+      </c>
+      <c r="D80" t="n">
+        <v>-0.2491065776143234</v>
+      </c>
+      <c r="E80" t="n">
+        <v>-4.538572400148866</v>
+      </c>
+      <c r="F80" t="n">
+        <v>-4.13113725292332</v>
+      </c>
+      <c r="G80" t="n">
+        <v>-7.281341609096803</v>
+      </c>
+      <c r="H80" t="n">
+        <v>-3.683252116661941</v>
+      </c>
+      <c r="I80" t="n">
+        <v>-13.70435482927903</v>
+      </c>
+      <c r="J80" t="n">
+        <v>-1.672895531954122</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B81" t="n">
+        <v>14.78034823942889</v>
+      </c>
+      <c r="C81" t="n">
+        <v>9.783510636627968</v>
+      </c>
+      <c r="D81" t="n">
+        <v>-0.1019456209410891</v>
+      </c>
+      <c r="E81" t="n">
+        <v>-3.546139181500126</v>
+      </c>
+      <c r="F81" t="n">
+        <v>-3.552412694655519</v>
+      </c>
+      <c r="G81" t="n">
+        <v>-6.888146119647407</v>
+      </c>
+      <c r="H81" t="n">
+        <v>-3.052909171134881</v>
+      </c>
+      <c r="I81" t="n">
+        <v>-11.72290897891374</v>
+      </c>
+      <c r="J81" t="n">
+        <v>-1.432001724950132</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B82" t="n">
+        <v>14.80675885378843</v>
+      </c>
+      <c r="C82" t="n">
+        <v>9.894614810739302</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0.506749691281287</v>
+      </c>
+      <c r="E82" t="n">
+        <v>-5.7393153121393</v>
+      </c>
+      <c r="F82" t="n">
+        <v>-3.445689196760248</v>
+      </c>
+      <c r="G82" t="n">
+        <v>-7.885498317840176</v>
+      </c>
+      <c r="H82" t="n">
+        <v>-2.913602782744853</v>
+      </c>
+      <c r="I82" t="n">
+        <v>-12.41387736451633</v>
+      </c>
+      <c r="J82" t="n">
+        <v>-1.263595932829914</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B83" t="n">
+        <v>14.655645961177</v>
+      </c>
+      <c r="C83" t="n">
+        <v>9.635511948738333</v>
+      </c>
+      <c r="D83" t="n">
+        <v>1.460671501257519</v>
+      </c>
+      <c r="E83" t="n">
+        <v>-5.558908537712642</v>
+      </c>
+      <c r="F83" t="n">
+        <v>-2.553346849752145</v>
+      </c>
+      <c r="G83" t="n">
+        <v>-7.563511102694441</v>
+      </c>
+      <c r="H83" t="n">
+        <v>-1.97696970540262</v>
+      </c>
+      <c r="I83" t="n">
+        <v>-11.34461988398101</v>
+      </c>
+      <c r="J83" t="n">
+        <v>-0.462134698829156</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B84" t="n">
+        <v>14.68207856730978</v>
+      </c>
+      <c r="C84" t="n">
+        <v>9.63558311523574</v>
+      </c>
+      <c r="D84" t="n">
+        <v>0.3754283347773305</v>
+      </c>
+      <c r="E84" t="n">
+        <v>-4.842999289582898</v>
+      </c>
+      <c r="F84" t="n">
+        <v>-3.438564208517317</v>
+      </c>
+      <c r="G84" t="n">
+        <v>-7.288312645342142</v>
+      </c>
+      <c r="H84" t="n">
+        <v>-2.943495606990662</v>
+      </c>
+      <c r="I84" t="n">
+        <v>-12.36715243182851</v>
+      </c>
+      <c r="J84" t="n">
+        <v>-1.21057129137471</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B85" t="n">
+        <v>14.98297962645542</v>
+      </c>
+      <c r="C85" t="n">
+        <v>10.06825119210434</v>
+      </c>
+      <c r="D85" t="n">
+        <v>2.063873740802449</v>
+      </c>
+      <c r="E85" t="n">
+        <v>-3.111113649518185</v>
+      </c>
+      <c r="F85" t="n">
+        <v>-1.64493793929409</v>
+      </c>
+      <c r="G85" t="n">
+        <v>-4.47940159354918</v>
+      </c>
+      <c r="H85" t="n">
+        <v>-1.305351573338812</v>
+      </c>
+      <c r="I85" t="n">
+        <v>-10.90166581512292</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0.6642975447069988</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B86" t="n">
+        <v>15.09507812461639</v>
+      </c>
+      <c r="C86" t="n">
+        <v>10.26619179262225</v>
+      </c>
+      <c r="D86" t="n">
+        <v>2.219108891821278</v>
+      </c>
+      <c r="E86" t="n">
+        <v>-4.537899269445709</v>
+      </c>
+      <c r="F86" t="n">
+        <v>-1.614531255306491</v>
+      </c>
+      <c r="G86" t="n">
+        <v>-5.809231966137929</v>
+      </c>
+      <c r="H86" t="n">
+        <v>-1.155436070768756</v>
+      </c>
+      <c r="I86" t="n">
+        <v>-10.38370776272435</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0.4761400597816969</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B87" t="n">
+        <v>14.97164884831495</v>
+      </c>
+      <c r="C87" t="n">
+        <v>10.0811710210642</v>
+      </c>
+      <c r="D87" t="n">
+        <v>1.099267272936277</v>
+      </c>
+      <c r="E87" t="n">
+        <v>-4.000628404216957</v>
+      </c>
+      <c r="F87" t="n">
+        <v>-2.424852310571561</v>
+      </c>
+      <c r="G87" t="n">
+        <v>-6.019866852411283</v>
+      </c>
+      <c r="H87" t="n">
+        <v>-1.977781254230233</v>
+      </c>
+      <c r="I87" t="n">
+        <v>-10.65092821480261</v>
+      </c>
+      <c r="J87" t="n">
+        <v>-0.3899661226759969</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D87"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>month_count</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>first_month</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>last_month</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1940</v>
+      </c>
+      <c r="B2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1941</v>
+      </c>
+      <c r="B3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1942</v>
+      </c>
+      <c r="B4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1943</v>
+      </c>
+      <c r="B5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1944</v>
+      </c>
+      <c r="B6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1945</v>
+      </c>
+      <c r="B7" t="n">
+        <v>12</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1946</v>
+      </c>
+      <c r="B8" t="n">
+        <v>12</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1947</v>
+      </c>
+      <c r="B9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1948</v>
+      </c>
+      <c r="B10" t="n">
+        <v>12</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1949</v>
+      </c>
+      <c r="B11" t="n">
+        <v>12</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1950</v>
+      </c>
+      <c r="B12" t="n">
+        <v>12</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1951</v>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1952</v>
+      </c>
+      <c r="B14" t="n">
+        <v>12</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1953</v>
+      </c>
+      <c r="B15" t="n">
+        <v>12</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>1954</v>
+      </c>
+      <c r="B16" t="n">
+        <v>12</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>1955</v>
+      </c>
+      <c r="B17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>1956</v>
+      </c>
+      <c r="B18" t="n">
+        <v>12</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1957</v>
+      </c>
+      <c r="B19" t="n">
+        <v>12</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1958</v>
+      </c>
+      <c r="B20" t="n">
+        <v>12</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>1959</v>
+      </c>
+      <c r="B21" t="n">
+        <v>12</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1960</v>
+      </c>
+      <c r="B22" t="n">
+        <v>12</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>1961</v>
+      </c>
+      <c r="B23" t="n">
+        <v>12</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>1962</v>
+      </c>
+      <c r="B24" t="n">
+        <v>12</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>1963</v>
+      </c>
+      <c r="B25" t="n">
+        <v>12</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>1964</v>
+      </c>
+      <c r="B26" t="n">
+        <v>12</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>1965</v>
+      </c>
+      <c r="B27" t="n">
+        <v>12</v>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>1966</v>
+      </c>
+      <c r="B28" t="n">
+        <v>12</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>1967</v>
+      </c>
+      <c r="B29" t="n">
+        <v>12</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>1968</v>
+      </c>
+      <c r="B30" t="n">
+        <v>12</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>1969</v>
+      </c>
+      <c r="B31" t="n">
+        <v>12</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>1970</v>
+      </c>
+      <c r="B32" t="n">
+        <v>12</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>1971</v>
+      </c>
+      <c r="B33" t="n">
+        <v>12</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>1972</v>
+      </c>
+      <c r="B34" t="n">
+        <v>12</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>1973</v>
+      </c>
+      <c r="B35" t="n">
+        <v>12</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>1974</v>
+      </c>
+      <c r="B36" t="n">
+        <v>12</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>1975</v>
+      </c>
+      <c r="B37" t="n">
+        <v>12</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>1976</v>
+      </c>
+      <c r="B38" t="n">
+        <v>12</v>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>1977</v>
+      </c>
+      <c r="B39" t="n">
+        <v>12</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>1978</v>
+      </c>
+      <c r="B40" t="n">
+        <v>12</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>1979</v>
+      </c>
+      <c r="B41" t="n">
+        <v>12</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>1980</v>
+      </c>
+      <c r="B42" t="n">
+        <v>12</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>1981</v>
+      </c>
+      <c r="B43" t="n">
+        <v>12</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>1982</v>
+      </c>
+      <c r="B44" t="n">
+        <v>12</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>1983</v>
+      </c>
+      <c r="B45" t="n">
+        <v>12</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>1984</v>
+      </c>
+      <c r="B46" t="n">
+        <v>12</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>1985</v>
+      </c>
+      <c r="B47" t="n">
+        <v>12</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>1986</v>
+      </c>
+      <c r="B48" t="n">
+        <v>12</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>1987</v>
+      </c>
+      <c r="B49" t="n">
+        <v>12</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>1988</v>
+      </c>
+      <c r="B50" t="n">
+        <v>12</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>1989</v>
+      </c>
+      <c r="B51" t="n">
+        <v>12</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>1990</v>
+      </c>
+      <c r="B52" t="n">
+        <v>12</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>1991</v>
+      </c>
+      <c r="B53" t="n">
+        <v>12</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>1992</v>
+      </c>
+      <c r="B54" t="n">
+        <v>12</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>1993</v>
+      </c>
+      <c r="B55" t="n">
+        <v>12</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>1994</v>
+      </c>
+      <c r="B56" t="n">
+        <v>12</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>1995</v>
+      </c>
+      <c r="B57" t="n">
+        <v>12</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>1996</v>
+      </c>
+      <c r="B58" t="n">
+        <v>12</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>1997</v>
+      </c>
+      <c r="B59" t="n">
+        <v>12</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>1998</v>
+      </c>
+      <c r="B60" t="n">
+        <v>12</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>1999</v>
+      </c>
+      <c r="B61" t="n">
+        <v>12</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B62" t="n">
+        <v>12</v>
+      </c>
+      <c r="C62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>2001</v>
+      </c>
+      <c r="B63" t="n">
+        <v>12</v>
+      </c>
+      <c r="C63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B64" t="n">
+        <v>12</v>
+      </c>
+      <c r="C64" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B65" t="n">
+        <v>12</v>
+      </c>
+      <c r="C65" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B66" t="n">
+        <v>12</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B67" t="n">
+        <v>12</v>
+      </c>
+      <c r="C67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B68" t="n">
+        <v>12</v>
+      </c>
+      <c r="C68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B69" t="n">
+        <v>12</v>
+      </c>
+      <c r="C69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B70" t="n">
+        <v>12</v>
+      </c>
+      <c r="C70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B71" t="n">
+        <v>12</v>
+      </c>
+      <c r="C71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B72" t="n">
+        <v>12</v>
+      </c>
+      <c r="C72" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B73" t="n">
+        <v>12</v>
+      </c>
+      <c r="C73" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B74" t="n">
+        <v>12</v>
+      </c>
+      <c r="C74" t="n">
+        <v>1</v>
+      </c>
+      <c r="D74" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B75" t="n">
+        <v>12</v>
+      </c>
+      <c r="C75" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B76" t="n">
+        <v>12</v>
+      </c>
+      <c r="C76" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B77" t="n">
+        <v>12</v>
+      </c>
+      <c r="C77" t="n">
+        <v>1</v>
+      </c>
+      <c r="D77" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B78" t="n">
+        <v>12</v>
+      </c>
+      <c r="C78" t="n">
+        <v>1</v>
+      </c>
+      <c r="D78" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B79" t="n">
+        <v>12</v>
+      </c>
+      <c r="C79" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B80" t="n">
+        <v>12</v>
+      </c>
+      <c r="C80" t="n">
+        <v>1</v>
+      </c>
+      <c r="D80" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B81" t="n">
+        <v>12</v>
+      </c>
+      <c r="C81" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B82" t="n">
+        <v>12</v>
+      </c>
+      <c r="C82" t="n">
+        <v>1</v>
+      </c>
+      <c r="D82" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B83" t="n">
+        <v>12</v>
+      </c>
+      <c r="C83" t="n">
+        <v>1</v>
+      </c>
+      <c r="D83" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B84" t="n">
+        <v>12</v>
+      </c>
+      <c r="C84" t="n">
+        <v>1</v>
+      </c>
+      <c r="D84" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B85" t="n">
+        <v>12</v>
+      </c>
+      <c r="C85" t="n">
+        <v>1</v>
+      </c>
+      <c r="D85" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B86" t="n">
+        <v>12</v>
+      </c>
+      <c r="C86" t="n">
+        <v>1</v>
+      </c>
+      <c r="D86" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B87" t="n">
+        <v>12</v>
+      </c>
+      <c r="C87" t="n">
+        <v>1</v>
+      </c>
+      <c r="D87" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update climate indicator methods and About data text
</commit_message>
<xml_diff>
--- a/data/tables/northern_warming/tables/northwest_territories_warming_tables.xlsx
+++ b/data/tables/northern_warming/tables/northwest_territories_warming_tables.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Average comparison report" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Average comparison full" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faster areas report" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faster areas full" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annual reference series" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Year completeness" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Average comparison report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Average comparison full" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Faster areas report" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Faster areas full" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Annual reference series" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Year completeness" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,16 +22,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,21 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,37 +422,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Start year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>End year</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Northwest Territories warming rate (°C/decade)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Compared with global average</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Compared with global land</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Compared with southern Canada</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Compared with rest of Canada</t>
         </is>
@@ -478,7 +466,7 @@
         <v>2025</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2638805455586553</v>
+        <v>0.2638805455586551</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -509,7 +497,7 @@
         <v>2025</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3672839573063428</v>
+        <v>0.3672839573063446</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -540,7 +528,7 @@
         <v>2025</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4360245424264593</v>
+        <v>0.4360245424264594</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -602,7 +590,7 @@
         <v>2025</v>
       </c>
       <c r="C6" t="n">
-        <v>0.4795372483656996</v>
+        <v>0.479537248365705</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -633,7 +621,7 @@
         <v>2025</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5415477130413764</v>
+        <v>0.5415477130413753</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -671,57 +659,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Start year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>End year</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Northwest Territories warming rate (°C/decade)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Compared with global average</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Compared with global land</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Compared with southern Canada</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Compared with rest of Canada</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Global average rate (°C/decade)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Global land rate (°C/decade)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Southern Canada rate (°C/decade)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Rest of Canada rate (°C/decade)</t>
         </is>
@@ -735,7 +723,7 @@
         <v>2025</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2638805455586553</v>
+        <v>0.2638805455586551</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -761,7 +749,7 @@
         <v>0.1420527509547941</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2208353673690072</v>
+        <v>0.2208353673690087</v>
       </c>
       <c r="J2" t="n">
         <v>0.2193122683420462</v>
@@ -778,7 +766,7 @@
         <v>2025</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3672839573063428</v>
+        <v>0.3672839573063446</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -801,16 +789,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.1648486220011619</v>
+        <v>0.1648486220011625</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2570259324213248</v>
+        <v>0.2570259324213272</v>
       </c>
       <c r="J3" t="n">
         <v>0.2799826390854742</v>
       </c>
       <c r="K3" t="n">
-        <v>0.3070893001596213</v>
+        <v>0.3070893001596218</v>
       </c>
     </row>
     <row r="4">
@@ -821,7 +809,7 @@
         <v>2025</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4360245424264593</v>
+        <v>0.4360245424264594</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -847,7 +835,7 @@
         <v>0.1874950696370267</v>
       </c>
       <c r="I4" t="n">
-        <v>0.2897269249773123</v>
+        <v>0.2897269249773138</v>
       </c>
       <c r="J4" t="n">
         <v>0.325175709998213</v>
@@ -887,10 +875,10 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.2128004446215391</v>
+        <v>0.2128004446215388</v>
       </c>
       <c r="I5" t="n">
-        <v>0.3280053462325782</v>
+        <v>0.3280053462325799</v>
       </c>
       <c r="J5" t="n">
         <v>0.375455574822453</v>
@@ -907,7 +895,7 @@
         <v>2025</v>
       </c>
       <c r="C6" t="n">
-        <v>0.4795372483656996</v>
+        <v>0.479537248365705</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -930,16 +918,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.213408810851062</v>
+        <v>0.2134088108510637</v>
       </c>
       <c r="I6" t="n">
-        <v>0.3343533519136058</v>
+        <v>0.3343533519136107</v>
       </c>
       <c r="J6" t="n">
-        <v>0.3429550470459525</v>
+        <v>0.3429550470459552</v>
       </c>
       <c r="K6" t="n">
-        <v>0.4090867065865657</v>
+        <v>0.40908670658657</v>
       </c>
     </row>
     <row r="7">
@@ -950,7 +938,7 @@
         <v>2025</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5415477130413764</v>
+        <v>0.5415477130413753</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -973,16 +961,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.2474403282590529</v>
+        <v>0.247440328259056</v>
       </c>
       <c r="I7" t="n">
-        <v>0.3762561489730054</v>
+        <v>0.3762561489730121</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4239276655602184</v>
+        <v>0.4239276655602218</v>
       </c>
       <c r="K7" t="n">
-        <v>0.4944605489941047</v>
+        <v>0.4944605489941079</v>
       </c>
     </row>
   </sheetData>
@@ -1000,37 +988,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Start year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>End year</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Fastest-warming areas in Northwest Territories</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Compared with global average</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Compared with global land</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Compared with southern Canada</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Compared with rest of Canada</t>
         </is>
@@ -1237,62 +1225,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Start year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>End year</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Fastest-warming areas in Northwest Territories</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Compared with global average</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Compared with global land</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Compared with southern Canada</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Compared with rest of Canada</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Global average rate (°C/decade)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Global land rate (°C/decade)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Southern Canada rate (°C/decade)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Rest of Canada rate (°C/decade)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Grid-cell percentile used</t>
         </is>
@@ -1332,7 +1320,7 @@
         <v>0.1420527509547941</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2208353673690072</v>
+        <v>0.2208353673690087</v>
       </c>
       <c r="J2" t="n">
         <v>0.2193122683420462</v>
@@ -1375,16 +1363,16 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.1648486220011619</v>
+        <v>0.1648486220011625</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2570259324213248</v>
+        <v>0.2570259324213272</v>
       </c>
       <c r="J3" t="n">
         <v>0.2799826390854742</v>
       </c>
       <c r="K3" t="n">
-        <v>0.3070893001596213</v>
+        <v>0.3070893001596218</v>
       </c>
       <c r="L3" t="n">
         <v>95</v>
@@ -1424,7 +1412,7 @@
         <v>0.1874950696370267</v>
       </c>
       <c r="I4" t="n">
-        <v>0.2897269249773123</v>
+        <v>0.2897269249773138</v>
       </c>
       <c r="J4" t="n">
         <v>0.325175709998213</v>
@@ -1467,10 +1455,10 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.2128004446215391</v>
+        <v>0.2128004446215388</v>
       </c>
       <c r="I5" t="n">
-        <v>0.3280053462325782</v>
+        <v>0.3280053462325799</v>
       </c>
       <c r="J5" t="n">
         <v>0.375455574822453</v>
@@ -1513,16 +1501,16 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.213408810851062</v>
+        <v>0.2134088108510637</v>
       </c>
       <c r="I6" t="n">
-        <v>0.3343533519136058</v>
+        <v>0.3343533519136107</v>
       </c>
       <c r="J6" t="n">
-        <v>0.3429550470459525</v>
+        <v>0.3429550470459552</v>
       </c>
       <c r="K6" t="n">
-        <v>0.4090867065865657</v>
+        <v>0.40908670658657</v>
       </c>
       <c r="L6" t="n">
         <v>95</v>
@@ -1559,16 +1547,16 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.2474403282590529</v>
+        <v>0.247440328259056</v>
       </c>
       <c r="I7" t="n">
-        <v>0.3762561489730054</v>
+        <v>0.3762561489730121</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4239276655602184</v>
+        <v>0.4239276655602218</v>
       </c>
       <c r="K7" t="n">
-        <v>0.4944605489941047</v>
+        <v>0.4944605489941079</v>
       </c>
       <c r="L7" t="n">
         <v>95</v>
@@ -1589,52 +1577,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Global average</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Global land</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Southern Canada</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Yukon</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Rest of Canada excluding Yukon</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Northwest Territories</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Rest of Canada excluding Northwest Territories</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Nunavut</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Rest of Canada excluding Nunavut</t>
         </is>
@@ -1648,7 +1636,7 @@
         <v>13.69043057564458</v>
       </c>
       <c r="C2" t="n">
-        <v>8.011690884027798</v>
+        <v>8.011690884027843</v>
       </c>
       <c r="D2" t="n">
         <v>-0.3326529592866357</v>
@@ -1680,7 +1668,7 @@
         <v>13.73878407089074</v>
       </c>
       <c r="C3" t="n">
-        <v>8.183946255132463</v>
+        <v>8.18394625513251</v>
       </c>
       <c r="D3" t="n">
         <v>-0.1905575050200881</v>
@@ -1712,7 +1700,7 @@
         <v>13.64891403451929</v>
       </c>
       <c r="C4" t="n">
-        <v>8.109579213069086</v>
+        <v>8.109579213069132</v>
       </c>
       <c r="D4" t="n">
         <v>-0.2103798882965486</v>
@@ -1744,7 +1732,7 @@
         <v>13.65366753361602</v>
       </c>
       <c r="C5" t="n">
-        <v>8.185407421028536</v>
+        <v>8.185407421028582</v>
       </c>
       <c r="D5" t="n">
         <v>-0.3772654547579293</v>
@@ -1776,7 +1764,7 @@
         <v>13.84095510596814</v>
       </c>
       <c r="C6" t="n">
-        <v>8.41790385075349</v>
+        <v>8.417903850753538</v>
       </c>
       <c r="D6" t="n">
         <v>0.4350702945745796</v>
@@ -1808,7 +1796,7 @@
         <v>13.7070656102983</v>
       </c>
       <c r="C7" t="n">
-        <v>8.106175190026693</v>
+        <v>8.10617519002674</v>
       </c>
       <c r="D7" t="n">
         <v>-1.153032981796486</v>
@@ -1840,7 +1828,7 @@
         <v>13.7090479413186</v>
       </c>
       <c r="C8" t="n">
-        <v>8.185659112404654</v>
+        <v>8.1856591124047</v>
       </c>
       <c r="D8" t="n">
         <v>-0.79323259784954</v>
@@ -1872,7 +1860,7 @@
         <v>13.75378213968676</v>
       </c>
       <c r="C9" t="n">
-        <v>8.236751371071195</v>
+        <v>8.236751371071241</v>
       </c>
       <c r="D9" t="n">
         <v>-0.6510887934858871</v>
@@ -1904,7 +1892,7 @@
         <v>13.68855663720653</v>
       </c>
       <c r="C10" t="n">
-        <v>8.176407852228916</v>
+        <v>8.176407852228962</v>
       </c>
       <c r="D10" t="n">
         <v>-0.8170015965818799</v>
@@ -1936,7 +1924,7 @@
         <v>13.72586943551582</v>
       </c>
       <c r="C11" t="n">
-        <v>8.190172609171192</v>
+        <v>8.190172609171238</v>
       </c>
       <c r="D11" t="n">
         <v>-1.03165884283921</v>
@@ -1968,7 +1956,7 @@
         <v>13.61467633330517</v>
       </c>
       <c r="C12" t="n">
-        <v>7.935410504753428</v>
+        <v>7.935410504753474</v>
       </c>
       <c r="D12" t="n">
         <v>-2.177027189220774</v>
@@ -2000,7 +1988,7 @@
         <v>13.74845288205021</v>
       </c>
       <c r="C13" t="n">
-        <v>8.149450338215479</v>
+        <v>8.149450338215525</v>
       </c>
       <c r="D13" t="n">
         <v>-1.346006348084203</v>
@@ -2032,7 +2020,7 @@
         <v>13.72560247225752</v>
       </c>
       <c r="C14" t="n">
-        <v>8.035272161708857</v>
+        <v>8.035272161708903</v>
       </c>
       <c r="D14" t="n">
         <v>0.1722462764292237</v>
@@ -2064,7 +2052,7 @@
         <v>13.80752023492195</v>
       </c>
       <c r="C15" t="n">
-        <v>8.334412993306447</v>
+        <v>8.334412993306495</v>
       </c>
       <c r="D15" t="n">
         <v>0.2347795141871966</v>
@@ -2096,7 +2084,7 @@
         <v>13.61034425644664</v>
       </c>
       <c r="C16" t="n">
-        <v>8.049068671152671</v>
+        <v>8.049068671152718</v>
       </c>
       <c r="D16" t="n">
         <v>-0.6628160976511045</v>
@@ -2128,7 +2116,7 @@
         <v>13.59340965381186</v>
       </c>
       <c r="C17" t="n">
-        <v>8.14187734084639</v>
+        <v>8.141877340846435</v>
       </c>
       <c r="D17" t="n">
         <v>-0.6810330503840414</v>
@@ -2160,7 +2148,7 @@
         <v>13.52870770667274</v>
       </c>
       <c r="C18" t="n">
-        <v>7.849739390896374</v>
+        <v>7.849739390896418</v>
       </c>
       <c r="D18" t="n">
         <v>-1.385824290000767</v>
@@ -2192,7 +2180,7 @@
         <v>13.78207114754643</v>
       </c>
       <c r="C19" t="n">
-        <v>8.225985666889731</v>
+        <v>8.225985666889777</v>
       </c>
       <c r="D19" t="n">
         <v>-0.7677594865095184</v>
@@ -2224,7 +2212,7 @@
         <v>13.84805935178077</v>
       </c>
       <c r="C20" t="n">
-        <v>8.380354078559543</v>
+        <v>8.380354078559591</v>
       </c>
       <c r="D20" t="n">
         <v>-0.02886261013903971</v>
@@ -2256,7 +2244,7 @@
         <v>13.81318674584848</v>
       </c>
       <c r="C21" t="n">
-        <v>8.323354789294006</v>
+        <v>8.323354789294052</v>
       </c>
       <c r="D21" t="n">
         <v>-0.9445410986697892</v>
@@ -2288,7 +2276,7 @@
         <v>13.76304280509798</v>
       </c>
       <c r="C22" t="n">
-        <v>8.172513567636624</v>
+        <v>8.17251356763667</v>
       </c>
       <c r="D22" t="n">
         <v>-0.3097222048625001</v>
@@ -2320,7 +2308,7 @@
         <v>13.84279138886267</v>
       </c>
       <c r="C23" t="n">
-        <v>8.376774708212775</v>
+        <v>8.376774708212823</v>
       </c>
       <c r="D23" t="n">
         <v>-0.2117103289607526</v>
@@ -2352,7 +2340,7 @@
         <v>13.78246811576126</v>
       </c>
       <c r="C24" t="n">
-        <v>8.325135007353035</v>
+        <v>8.325135007353083</v>
       </c>
       <c r="D24" t="n">
         <v>-0.8072732988162884</v>
@@ -2384,7 +2372,7 @@
         <v>13.81946226871661</v>
       </c>
       <c r="C25" t="n">
-        <v>8.415733425862536</v>
+        <v>8.415733425862582</v>
       </c>
       <c r="D25" t="n">
         <v>-0.5155131683942684</v>
@@ -2416,7 +2404,7 @@
         <v>13.60333128437458</v>
       </c>
       <c r="C26" t="n">
-        <v>8.023429813772184</v>
+        <v>8.023429813772228</v>
       </c>
       <c r="D26" t="n">
         <v>-1.007449437201353</v>
@@ -2448,7 +2436,7 @@
         <v>13.67094742700516</v>
       </c>
       <c r="C27" t="n">
-        <v>8.152862461762012</v>
+        <v>8.152862461762059</v>
       </c>
       <c r="D27" t="n">
         <v>-1.50479333529286</v>
@@ -2480,7 +2468,7 @@
         <v>13.74815768230339</v>
       </c>
       <c r="C28" t="n">
-        <v>8.224824069412861</v>
+        <v>8.224824069412907</v>
       </c>
       <c r="D28" t="n">
         <v>-0.8201873242751556</v>
@@ -2512,7 +2500,7 @@
         <v>13.7634132530287</v>
       </c>
       <c r="C29" t="n">
-        <v>8.262825607848763</v>
+        <v>8.262825607848809</v>
       </c>
       <c r="D29" t="n">
         <v>-1.184187030358838</v>
@@ -2544,7 +2532,7 @@
         <v>13.695035187117</v>
       </c>
       <c r="C30" t="n">
-        <v>8.123353720947794</v>
+        <v>8.12335372094784</v>
       </c>
       <c r="D30" t="n">
         <v>-0.5450112004398701</v>
@@ -2576,7 +2564,7 @@
         <v>13.8312038334572</v>
       </c>
       <c r="C31" t="n">
-        <v>8.213444446430842</v>
+        <v>8.213444446430888</v>
       </c>
       <c r="D31" t="n">
         <v>-0.4802128268041829</v>
@@ -2608,7 +2596,7 @@
         <v>13.80381375678246</v>
       </c>
       <c r="C32" t="n">
-        <v>8.344194338117621</v>
+        <v>8.344194338117669</v>
       </c>
       <c r="D32" t="n">
         <v>-0.9403054837497881</v>
@@ -2640,7 +2628,7 @@
         <v>13.65070870843836</v>
       </c>
       <c r="C33" t="n">
-        <v>8.251643007445134</v>
+        <v>8.25164300744518</v>
       </c>
       <c r="D33" t="n">
         <v>-0.6759595449608697</v>
@@ -2672,7 +2660,7 @@
         <v>13.78198341342426</v>
       </c>
       <c r="C34" t="n">
-        <v>8.150958367031723</v>
+        <v>8.15095836703177</v>
       </c>
       <c r="D34" t="n">
         <v>-2.566915333819982</v>
@@ -2704,7 +2692,7 @@
         <v>13.88761343950328</v>
       </c>
       <c r="C35" t="n">
-        <v>8.589287371277686</v>
+        <v>8.589287371277736</v>
       </c>
       <c r="D35" t="n">
         <v>0.07229780815960817</v>
@@ -2736,7 +2724,7 @@
         <v>13.61420722376732</v>
       </c>
       <c r="C36" t="n">
-        <v>8.002236108952145</v>
+        <v>8.002236108952189</v>
       </c>
       <c r="D36" t="n">
         <v>-1.237721589227154</v>
@@ -2768,7 +2756,7 @@
         <v>13.63716264439821</v>
       </c>
       <c r="C37" t="n">
-        <v>8.265033478330494</v>
+        <v>8.26503347833054</v>
       </c>
       <c r="D37" t="n">
         <v>-0.7736300103879947</v>
@@ -2800,7 +2788,7 @@
         <v>13.56440519112469</v>
       </c>
       <c r="C38" t="n">
-        <v>7.879184523090127</v>
+        <v>7.879184523090172</v>
       </c>
       <c r="D38" t="n">
         <v>-0.7226998836723107</v>
@@ -2832,7 +2820,7 @@
         <v>13.85508062118923</v>
       </c>
       <c r="C39" t="n">
-        <v>8.383890645727373</v>
+        <v>8.383890645727419</v>
       </c>
       <c r="D39" t="n">
         <v>0.2033718656115622</v>
@@ -2864,7 +2852,7 @@
         <v>13.79599116635706</v>
       </c>
       <c r="C40" t="n">
-        <v>8.247198056775574</v>
+        <v>8.24719805677562</v>
       </c>
       <c r="D40" t="n">
         <v>-1.246338815524421</v>
@@ -2896,7 +2884,7 @@
         <v>13.95342295070824</v>
       </c>
       <c r="C41" t="n">
-        <v>8.401263366793479</v>
+        <v>8.401263366793527</v>
       </c>
       <c r="D41" t="n">
         <v>-0.6732554052500564</v>
@@ -2928,7 +2916,7 @@
         <v>14.07790809274332</v>
       </c>
       <c r="C42" t="n">
-        <v>8.697190817270185</v>
+        <v>8.697190817270235</v>
       </c>
       <c r="D42" t="n">
         <v>-0.4842241006869986</v>
@@ -2960,7 +2948,7 @@
         <v>14.11629583112865</v>
       </c>
       <c r="C43" t="n">
-        <v>8.888912599967027</v>
+        <v>8.888912599967078</v>
       </c>
       <c r="D43" t="n">
         <v>1.210247003543447</v>
@@ -2992,7 +2980,7 @@
         <v>13.91712094370134</v>
       </c>
       <c r="C44" t="n">
-        <v>8.362596808060404</v>
+        <v>8.36259680806045</v>
       </c>
       <c r="D44" t="n">
         <v>-1.50289562012097</v>
@@ -3024,7 +3012,7 @@
         <v>14.11096790609288</v>
       </c>
       <c r="C45" t="n">
-        <v>8.738856444670766</v>
+        <v>8.738856444670816</v>
       </c>
       <c r="D45" t="n">
         <v>-0.1845328916807096</v>
@@ -3056,7 +3044,7 @@
         <v>13.89532993274377</v>
       </c>
       <c r="C46" t="n">
-        <v>8.375720439317485</v>
+        <v>8.375720439317533</v>
       </c>
       <c r="D46" t="n">
         <v>-0.2221425623810813</v>
@@ -3088,7 +3076,7 @@
         <v>13.85986580938163</v>
       </c>
       <c r="C47" t="n">
-        <v>8.326186326237247</v>
+        <v>8.326186326237295</v>
       </c>
       <c r="D47" t="n">
         <v>-0.8474040933769079</v>
@@ -3120,7 +3108,7 @@
         <v>13.94697218635512</v>
       </c>
       <c r="C48" t="n">
-        <v>8.529983752026428</v>
+        <v>8.529983752026476</v>
       </c>
       <c r="D48" t="n">
         <v>-0.2514886508334715</v>
@@ -3152,7 +3140,7 @@
         <v>14.10282603145438</v>
       </c>
       <c r="C49" t="n">
-        <v>8.700475228206267</v>
+        <v>8.700475228206317</v>
       </c>
       <c r="D49" t="n">
         <v>1.34994300806786</v>
@@ -3184,7 +3172,7 @@
         <v>14.13113825237433</v>
       </c>
       <c r="C50" t="n">
-        <v>8.907656175206741</v>
+        <v>8.907656175206791</v>
       </c>
       <c r="D50" t="n">
         <v>-0.04835242697436799</v>
@@ -3216,7 +3204,7 @@
         <v>14.01638740546175</v>
       </c>
       <c r="C51" t="n">
-        <v>8.65657060190965</v>
+        <v>8.656570601909698</v>
       </c>
       <c r="D51" t="n">
         <v>-0.9264306289894491</v>
@@ -3248,7 +3236,7 @@
         <v>14.24924986771015</v>
       </c>
       <c r="C52" t="n">
-        <v>8.974928186866773</v>
+        <v>8.974928186866824</v>
       </c>
       <c r="D52" t="n">
         <v>-0.4754288929981274</v>
@@ -3280,7 +3268,7 @@
         <v>14.19236932713923</v>
       </c>
       <c r="C53" t="n">
-        <v>8.885097619611615</v>
+        <v>8.885097619611667</v>
       </c>
       <c r="D53" t="n">
         <v>-0.0390618734019884</v>
@@ -3312,7 +3300,7 @@
         <v>13.95644895242778</v>
       </c>
       <c r="C54" t="n">
-        <v>8.470906583813663</v>
+        <v>8.470906583813711</v>
       </c>
       <c r="D54" t="n">
         <v>-0.7546456587878561</v>
@@ -3344,7 +3332,7 @@
         <v>14.00688804708349</v>
       </c>
       <c r="C55" t="n">
-        <v>8.583487742832272</v>
+        <v>8.583487742832322</v>
       </c>
       <c r="D55" t="n">
         <v>-0.4712216502193975</v>
@@ -3376,7 +3364,7 @@
         <v>14.04477926471139</v>
       </c>
       <c r="C56" t="n">
-        <v>8.755904775315386</v>
+        <v>8.755904775315436</v>
       </c>
       <c r="D56" t="n">
         <v>-0.3150391664258419</v>
@@ -3408,7 +3396,7 @@
         <v>14.21911714260189</v>
       </c>
       <c r="C57" t="n">
-        <v>9.044514844715234</v>
+        <v>9.044514844715286</v>
       </c>
       <c r="D57" t="n">
         <v>-0.2922674313945443</v>
@@ -3440,7 +3428,7 @@
         <v>14.08627927036392</v>
       </c>
       <c r="C58" t="n">
-        <v>8.692077179223393</v>
+        <v>8.692077179223443</v>
       </c>
       <c r="D58" t="n">
         <v>-1.150548652493746</v>
@@ -3472,7 +3460,7 @@
         <v>14.21396009353637</v>
       </c>
       <c r="C59" t="n">
-        <v>8.833450567413729</v>
+        <v>8.833450567413779</v>
       </c>
       <c r="D59" t="n">
         <v>-0.1847919496307432</v>
@@ -3504,7 +3492,7 @@
         <v>14.40097630563749</v>
       </c>
       <c r="C60" t="n">
-        <v>9.205549128702256</v>
+        <v>9.205549128702307</v>
       </c>
       <c r="D60" t="n">
         <v>1.378348984312762</v>
@@ -3536,7 +3524,7 @@
         <v>14.13149572585292</v>
       </c>
       <c r="C61" t="n">
-        <v>8.950350886701687</v>
+        <v>8.950350886701738</v>
       </c>
       <c r="D61" t="n">
         <v>1.195861211541586</v>
@@ -3568,7 +3556,7 @@
         <v>14.12251664054831</v>
       </c>
       <c r="C62" t="n">
-        <v>8.808146153756283</v>
+        <v>8.808146153756333</v>
       </c>
       <c r="D62" t="n">
         <v>-0.08135084802839247</v>
@@ -3600,7 +3588,7 @@
         <v>14.28915395293253</v>
       </c>
       <c r="C63" t="n">
-        <v>9.08596114694458</v>
+        <v>9.085961146944632</v>
       </c>
       <c r="D63" t="n">
         <v>1.239415280566746</v>
@@ -3632,7 +3620,7 @@
         <v>14.38501333826196</v>
       </c>
       <c r="C64" t="n">
-        <v>9.267174959257533</v>
+        <v>9.267174959257586</v>
       </c>
       <c r="D64" t="n">
         <v>-0.4576761390656653</v>
@@ -3664,7 +3652,7 @@
         <v>14.3728158769447</v>
       </c>
       <c r="C65" t="n">
-        <v>9.216521340150363</v>
+        <v>9.216521340150415</v>
       </c>
       <c r="D65" t="n">
         <v>0.2273824884112743</v>
@@ -3696,7 +3684,7 @@
         <v>14.30470323905453</v>
       </c>
       <c r="C66" t="n">
-        <v>9.026763455166556</v>
+        <v>9.026763455166607</v>
       </c>
       <c r="D66" t="n">
         <v>-0.2966044438257777</v>
@@ -3728,7 +3716,7 @@
         <v>14.47313817288972</v>
       </c>
       <c r="C67" t="n">
-        <v>9.43795712433538</v>
+        <v>9.437957124335433</v>
       </c>
       <c r="D67" t="n">
         <v>1.030610573884831</v>
@@ -3760,7 +3748,7 @@
         <v>14.42411520384602</v>
       </c>
       <c r="C68" t="n">
-        <v>9.286630563005993</v>
+        <v>9.286630563006046</v>
       </c>
       <c r="D68" t="n">
         <v>1.699621116550594</v>
@@ -3792,7 +3780,7 @@
         <v>14.41695814330639</v>
       </c>
       <c r="C69" t="n">
-        <v>9.472656279833451</v>
+        <v>9.472656279833505</v>
       </c>
       <c r="D69" t="n">
         <v>0.1891081808003666</v>
@@ -3824,7 +3812,7 @@
         <v>14.28106556295393</v>
       </c>
       <c r="C70" t="n">
-        <v>9.143188597309269</v>
+        <v>9.143188597309321</v>
       </c>
       <c r="D70" t="n">
         <v>-0.0898154995451273</v>
@@ -3856,7 +3844,7 @@
         <v>14.41565621438641</v>
       </c>
       <c r="C71" t="n">
-        <v>9.256013601363724</v>
+        <v>9.256013601363778</v>
       </c>
       <c r="D71" t="n">
         <v>-0.1047786439621025</v>
@@ -3888,7 +3876,7 @@
         <v>14.51001282645987</v>
       </c>
       <c r="C72" t="n">
-        <v>9.468710411827946</v>
+        <v>9.468710411827999</v>
       </c>
       <c r="D72" t="n">
         <v>2.038150291331934</v>
@@ -3920,7 +3908,7 @@
         <v>14.37030848032745</v>
       </c>
       <c r="C73" t="n">
-        <v>9.249171651857194</v>
+        <v>9.249171651857246</v>
       </c>
       <c r="D73" t="n">
         <v>0.6242405824896694</v>
@@ -3952,7 +3940,7 @@
         <v>14.41598237324642</v>
       </c>
       <c r="C74" t="n">
-        <v>9.248810252234385</v>
+        <v>9.248810252234437</v>
       </c>
       <c r="D74" t="n">
         <v>1.142947544559073</v>
@@ -3984,7 +3972,7 @@
         <v>14.44748933354398</v>
       </c>
       <c r="C75" t="n">
-        <v>9.387085708574924</v>
+        <v>9.387085708574977</v>
       </c>
       <c r="D75" t="n">
         <v>0.0987622897893656</v>
@@ -4016,7 +4004,7 @@
         <v>14.48824158723409</v>
       </c>
       <c r="C76" t="n">
-        <v>9.340143525392069</v>
+        <v>9.340143525392122</v>
       </c>
       <c r="D76" t="n">
         <v>-0.2222100116732272</v>
@@ -4048,7 +4036,7 @@
         <v>14.63674357729909</v>
       </c>
       <c r="C77" t="n">
-        <v>9.626736475286478</v>
+        <v>9.626736475286531</v>
       </c>
       <c r="D77" t="n">
         <v>0.6916255165401095</v>
@@ -4080,7 +4068,7 @@
         <v>14.81423450213943</v>
       </c>
       <c r="C78" t="n">
-        <v>9.834334388164306</v>
+        <v>9.834334388164361</v>
       </c>
       <c r="D78" t="n">
         <v>1.122079311476868</v>
@@ -4112,7 +4100,7 @@
         <v>14.72358098865754</v>
       </c>
       <c r="C79" t="n">
-        <v>9.695913720390354</v>
+        <v>9.69591372039041</v>
       </c>
       <c r="D79" t="n">
         <v>0.6232090945763307</v>
@@ -4144,7 +4132,7 @@
         <v>14.64448905881926</v>
       </c>
       <c r="C80" t="n">
-        <v>9.552322644933925</v>
+        <v>9.55232264493398</v>
       </c>
       <c r="D80" t="n">
         <v>-0.2491065776143234</v>
@@ -4176,7 +4164,7 @@
         <v>14.78034823942889</v>
       </c>
       <c r="C81" t="n">
-        <v>9.783510636627968</v>
+        <v>9.783510636628023</v>
       </c>
       <c r="D81" t="n">
         <v>-0.1019456209410891</v>
@@ -4208,7 +4196,7 @@
         <v>14.80675885378843</v>
       </c>
       <c r="C82" t="n">
-        <v>9.894614810739302</v>
+        <v>9.894614810739359</v>
       </c>
       <c r="D82" t="n">
         <v>0.506749691281287</v>
@@ -4240,7 +4228,7 @@
         <v>14.655645961177</v>
       </c>
       <c r="C83" t="n">
-        <v>9.635511948738333</v>
+        <v>9.635511948738388</v>
       </c>
       <c r="D83" t="n">
         <v>1.460671501257519</v>
@@ -4272,7 +4260,7 @@
         <v>14.68207856730978</v>
       </c>
       <c r="C84" t="n">
-        <v>9.63558311523574</v>
+        <v>9.635583115235795</v>
       </c>
       <c r="D84" t="n">
         <v>0.3754283347773305</v>
@@ -4304,7 +4292,7 @@
         <v>14.98297962645542</v>
       </c>
       <c r="C85" t="n">
-        <v>10.06825119210434</v>
+        <v>10.0682511921044</v>
       </c>
       <c r="D85" t="n">
         <v>2.063873740802449</v>
@@ -4336,7 +4324,7 @@
         <v>15.09507812461639</v>
       </c>
       <c r="C86" t="n">
-        <v>10.26619179262225</v>
+        <v>10.26619179262231</v>
       </c>
       <c r="D86" t="n">
         <v>2.219108891821278</v>
@@ -4368,7 +4356,7 @@
         <v>14.97164884831495</v>
       </c>
       <c r="C87" t="n">
-        <v>10.0811710210642</v>
+        <v>10.08117102106426</v>
       </c>
       <c r="D87" t="n">
         <v>1.099267272936277</v>
@@ -4403,26 +4391,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D87"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>month_count</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>first_month</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>last_month</t>
         </is>
@@ -5630,6 +5618,20 @@
       </c>
       <c r="D87" t="n">
         <v>12</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B88" t="n">
+        <v>6</v>
+      </c>
+      <c r="C88" t="n">
+        <v>1</v>
+      </c>
+      <c r="D88" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>